<commit_message>
Add data management plan JSON files for C-GEM and Gu Laboratory projects
- Created sample12.json for C-GEM Data Management Plan detailing data sharing, research products, data formats, access policies, and archival standards.
- Created sample13.json for Gu Laboratory's Data Management Plan focusing on proteomic data, biological materials, publications, archiving, and teaching curricula.
- Structured JSON files added to output directories for both projects, ensuring compliance with NSF guidelines and promoting open data sharing practices.
</commit_message>
<xml_diff>
--- a/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
+++ b/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
@@ -19,6 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample9" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample10" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample12" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample13" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C149"/>
+  <dimension ref="A1:C196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2974,6 +2976,805 @@
       <c r="C149" t="inlineStr">
         <is>
           <t>We will publish primary results expeditiously in peer-reviewed journals, supported by relevant data in the supplementary documents along with the published papers. Raw data supporting published papers will be made available to the public automatically by depositing the data to the open-access repository Figshare, and the web link will be provided in the published paper. The raw data will be properly annotated and detailed metadata that describes the content, format, organization of the raw data will also be provided to help interpret the raw data. If processed data is used in the publication, the processing procedure will be described in detail in the paper. We will provide full assistance in terms of raw data availability, data processing software and error analysis for other researchers to validate and reproduce our results. We will make peer-reviewed publications from this project all available to the public by depositing the accepted manuscripts to depositories like arXiv and PubMed Central.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>C-GEM: Plan for Data Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>This Data Management Plan has been prepared in accordance with guidelines from the NSF Division of Chemistry, “Advice to PIs on Data Management Plans,” and is consistent with the NSF Policy on Dissemination and Sharing of Research Results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Data Sharing Across Teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>The C-GEM team will store, share, disseminate, and archive data following well-established, open, effective, secure, and timely processes. At the core of our Data Management strategy is GEM-NET, a set of web tools that support virtual teamwork via a Google Team Drive that provides unlimited storage for presentations, documents, and other data, including the underlying data storage for our custom data management apps. These custom apps include: - Strains, which tracks the identity and transfer of strains and plasmids; - Protocols, which documents our laboratory procedures; and - Molecules (in progress), which houses information on the structures, synthesis, characterization, and team usage of C-GEM monomers. Future work will incorporate a “search by structure” capability to help users find monomers quickly even when the archive scales to thousands of entries. We will also develop a searchable archive of GEM-NET Laboratory Notebooks that document research and can be associated with specific records in our Protocols, Strains, and Molecules databases. All new team members will receive a GEM-NET orientation to help them become rapidly proficient in each of these tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>1. C-GEM Research Products</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>(A) Materials. C-GEM scientists will produce new chemical compounds, new biological reagents, and new bacterial strains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>(B) Experimental Data. Data will be collected from chemical synthesis procedures, biochemical, structural, and molecular biology experiments, and structural and functional characterization of C-GEM polymers. Such data include spectra, chromatograms, diffraction data, images, and results of properties analysis. Metadata will be generated describing the storage locations of chemical compounds, plasmids, and bacterial strains. We will also generate annotations of various sequence information (polymers, proteins, DNA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>(C) Software. We will generate software including custom GEM-NET apps written in Python, algorithms for the Rosetta molecular modeling software suite, and simulation programs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>(D) Other Products. We will generate experimental protocols and collect data on GEM-NET usage from component services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>(E) Education and Outreach Materials. Our broader impacts and public engagement activities will generate educational materials (syllabi, lectures, demonstrations, hands-on activities) and online content (videos, blog posts, podcasts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>(F) Evaluation Data. Our management and broader impact activities will generate assessments, narratives, and aggregated information about participants. Human subject protocols will be developed and submitted for IRB review/approval at each institution pending notice of award.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>2. Data Format</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Collected data will be formatted in several ways: (A) images as .tiff files; (B) experimental data as csv/Excel files or more specialized formats from the output of FACS, LC-MS, cryo-EM, etc.; and (C) laboratory protocols and notes, initially as pdfs or images scanned from lab notebooks, and then in a common GEM-NET Notebook format. Whenever possible, we will save data in machine-readable non-proprietary formats; in cases where that is not possible, we will provide images or extracted data to interested parties upon request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>3. Access to Data and Data Sharing Practices and Policies</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>(B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>(C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>(D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>(E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>(F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives. The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>(A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>(B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>5. Archival Storage Standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>(A) Timing. Data will be archived within 1 month of validation or upon publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>(B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>sample12</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>(C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Understanding the protein composition and dynamics of the nuclear envelope in plants</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t># DATA MANAGEMENT PLAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Proteomic Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Archiving and Dissemination</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Teaching Curricula</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>sample13</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Lectures, student presentations, data collection, training resources will be maintained online through the UC Berkeley bCourses course management system and backed up online through the unlimited cloud-based storage space offered by Google.</t>
         </is>
       </c>
     </row>
@@ -3408,6 +4209,630 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C-GEM: Plan for Data Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>This Data Management Plan has been prepared in accordance with guidelines from the NSF Division of Chemistry, “Advice to PIs on Data Management Plans,” and is consistent with the NSF Policy on Dissemination and Sharing of Research Results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Data Sharing Across Teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>The C-GEM team will store, share, disseminate, and archive data following well-established, open, effective, secure, and timely processes. At the core of our Data Management strategy is GEM-NET, a set of web tools that support virtual teamwork via a Google Team Drive that provides unlimited storage for presentations, documents, and other data, including the underlying data storage for our custom data management apps. These custom apps include: - Strains, which tracks the identity and transfer of strains and plasmids; - Protocols, which documents our laboratory procedures; and - Molecules (in progress), which houses information on the structures, synthesis, characterization, and team usage of C-GEM monomers. Future work will incorporate a “search by structure” capability to help users find monomers quickly even when the archive scales to thousands of entries. We will also develop a searchable archive of GEM-NET Laboratory Notebooks that document research and can be associated with specific records in our Protocols, Strains, and Molecules databases. All new team members will receive a GEM-NET orientation to help them become rapidly proficient in each of these tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1. C-GEM Research Products</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>(A) Materials. C-GEM scientists will produce new chemical compounds, new biological reagents, and new bacterial strains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>(B) Experimental Data. Data will be collected from chemical synthesis procedures, biochemical, structural, and molecular biology experiments, and structural and functional characterization of C-GEM polymers. Such data include spectra, chromatograms, diffraction data, images, and results of properties analysis. Metadata will be generated describing the storage locations of chemical compounds, plasmids, and bacterial strains. We will also generate annotations of various sequence information (polymers, proteins, DNA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>(C) Software. We will generate software including custom GEM-NET apps written in Python, algorithms for the Rosetta molecular modeling software suite, and simulation programs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>(D) Other Products. We will generate experimental protocols and collect data on GEM-NET usage from component services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>(E) Education and Outreach Materials. Our broader impacts and public engagement activities will generate educational materials (syllabi, lectures, demonstrations, hands-on activities) and online content (videos, blog posts, podcasts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>(F) Evaluation Data. Our management and broader impact activities will generate assessments, narratives, and aggregated information about participants. Human subject protocols will be developed and submitted for IRB review/approval at each institution pending notice of award.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2. Data Format</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Collected data will be formatted in several ways: (A) images as .tiff files; (B) experimental data as csv/Excel files or more specialized formats from the output of FACS, LC-MS, cryo-EM, etc.; and (C) laboratory protocols and notes, initially as pdfs or images scanned from lab notebooks, and then in a common GEM-NET Notebook format. Whenever possible, we will save data in machine-readable non-proprietary formats; in cases where that is not possible, we will provide images or extracted data to interested parties upon request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3. Access to Data and Data Sharing Practices and Policies</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>(B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>(C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>(D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>(E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>(F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives. The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>(A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>(B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>5. Archival Storage Standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>(A) Timing. Data will be archived within 1 month of validation or upon publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>(B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>question.text</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>(C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Understanding the protein composition and dynamics of the nuclear envelope in plants</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t># DATA MANAGEMENT PLAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Proteomic Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Publications</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Archiving and Dissemination</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Teaching Curricula</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lectures, student presentations, data collection, training resources will be maintained online through the UC Berkeley bCourses course management system and backed up online through the unlimited cloud-based storage space offered by Google.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Refactor JSON data structure in samples 12 and 13 to improve clarity and organization; update LightOn extractor to handle page text merging more effectively; adjust export notebook to reflect updated sample data and ensure accurate output.
</commit_message>
<xml_diff>
--- a/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
+++ b/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C196"/>
+  <dimension ref="A1:C194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3242,12 +3242,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines.</t>
+          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines. (B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs). (C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice. (D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website. (E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication. (F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
         </is>
       </c>
     </row>
@@ -3259,12 +3259,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>(B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs).</t>
+          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives</t>
         </is>
       </c>
     </row>
@@ -3276,12 +3276,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>(C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice.</t>
+          <t>The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan. (A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access. (B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
         </is>
       </c>
     </row>
@@ -3293,12 +3293,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>(D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website.</t>
+          <t>5. Archival Storage Standards</t>
         </is>
       </c>
     </row>
@@ -3310,87 +3310,87 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>(E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication.</t>
+          <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive. (A) Timing. Data will be archived within 1 month of validation or upon publication. (B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley. (C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>(F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
+          <t>Understanding the protein composition and dynamics of the nuclear envelope in plants</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives. The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan.</t>
+          <t>DATA MANAGEMENT PLAN</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>(A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access.</t>
+          <t>PI Gu</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>(B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
+          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -3400,14 +3400,14 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>5. Archival Storage Standards</t>
+          <t>Proteomic Data</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -3417,58 +3417,58 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive.</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>(A) Timing. Data will be archived within 1 month of validation or upon publication.</t>
+          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>(B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley.</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>(C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
+          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.</t>
         </is>
       </c>
     </row>
@@ -3480,12 +3480,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Understanding the protein composition and dynamics of the nuclear envelope in plants</t>
+          <t>Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t># DATA MANAGEMENT PLAN</t>
+          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
         </is>
       </c>
     </row>
@@ -3514,12 +3514,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
@@ -3531,12 +3531,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Proteomic Data</t>
+          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
         </is>
       </c>
     </row>
@@ -3548,12 +3548,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.</t>
+          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
         </is>
       </c>
     </row>
@@ -3582,12 +3582,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
+          <t>Publications</t>
         </is>
       </c>
     </row>
@@ -3599,12 +3599,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
+          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
         </is>
       </c>
     </row>
@@ -3633,12 +3633,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
@@ -3650,12 +3650,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Publications</t>
+          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
         </is>
       </c>
     </row>
@@ -3667,12 +3667,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no</t>
+          <t>Teaching Curricula</t>
         </is>
       </c>
     </row>
@@ -3684,12 +3684,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
@@ -3701,12 +3701,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Archiving and Dissemination</t>
+          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
         </is>
       </c>
     </row>
@@ -3718,12 +3718,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
@@ -3735,44 +3735,10 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
-        <is>
-          <t>Teaching Curricula</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
         <is>
           <t>Lectures, student presentations, data collection, training resources will be maintained online through the UC Berkeley bCourses course management system and backed up online through the unlimited cloud-based storage space offered by Google.</t>
         </is>
@@ -4215,7 +4181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4309,7 +4275,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4321,7 +4287,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4333,7 +4299,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4345,7 +4311,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4357,7 +4323,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4369,7 +4335,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4417,168 +4383,60 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines.</t>
+          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines. (B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs). (C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice. (D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website. (E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication. (F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>(B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs).</t>
+          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>(C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice.</t>
+          <t>The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan. (A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access. (B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>(D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website.</t>
+          <t>5. Archival Storage Standards</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>(E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>question.text</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>(F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives. The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>question.text</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>(A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>question.text</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>(B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>5. Archival Storage Standards</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>question.text</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>(A) Timing. Data will be archived within 1 month of validation or upon publication.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>question.text</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>(B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>question.text</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>(C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
+          <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive. (A) Timing. Data will be archived within 1 month of validation or upon publication. (B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley. (C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
         </is>
       </c>
     </row>
@@ -4593,7 +4451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4632,67 +4490,67 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t># DATA MANAGEMENT PLAN</t>
+          <t>DATA MANAGEMENT PLAN</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
+          <t>PI Gu</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Proteomic Data</t>
+          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
+          <t>Proteomic Data</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
+          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
         </is>
       </c>
     </row>
@@ -4704,19 +4562,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
+          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.</t>
         </is>
       </c>
     </row>
@@ -4728,7 +4586,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
+          <t>Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
         </is>
       </c>
     </row>
@@ -4740,7 +4598,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Publications</t>
+          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
         </is>
       </c>
     </row>
@@ -4752,19 +4610,19 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
+          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4646,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
+          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4658,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Teaching Curricula</t>
+          <t>Publications</t>
         </is>
       </c>
     </row>
@@ -4812,17 +4670,101 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
+        <is>
+          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Archiving and Dissemination</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Teaching Curricula</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>section.description</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>section.title</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Archiving and Dissemination</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>answer.text</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>Lectures, student presentations, data collection, training resources will be maintained online through the UC Berkeley bCourses course management system and backed up online through the unlimited cloud-based storage space offered by Google.</t>
         </is>

</xml_diff>

<commit_message>
Enhance Excel export notebook to merge consecutive repeated labels and update documentation
</commit_message>
<xml_diff>
--- a/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
+++ b/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C194"/>
+  <dimension ref="A1:C169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1105,7 +1105,9 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>All data pertaining to any published work will be made available to any person on request. Numerical published data as well as the original raw data files will be freely accessible either as supplementary data files included with published papers, or as files posted on the web sites of the laboratories in the Center. Additional data or programs required by third parties will be provided on request. Data that may support intellectual property claims will be published only after we seek advice from the Northwestern Innovation and New Ventures Office (INVO). Such advice will be sought in a timely manner. Otherwise, there are no restrictions on who will be allowed to use the data generated after publishing is complete, provided that the requester acknowledges the original work. A requester can use data output of our work, provided guidelines by the publisher for use of published data are followed.</t>
+          <t>All data pertaining to any published work will be made available to any person on request. Numerical published data as well as the original raw data files will be freely accessible either as supplementary data files included with published papers, or as files posted on the web sites of the laboratories in the Center. Additional data or programs required by third parties will be provided on request. Data that may support intellectual property claims will be published only after we seek advice from the Northwestern Innovation and New Ventures Office (INVO). Such advice will be sought in a timely manner. Otherwise, there are no restrictions on who will be allowed to use the data generated after publishing is complete, provided that the requester acknowledges the original work. A requester can use data output of our work, provided guidelines by the publisher for use of published data are followed.
+Electronic files are stored on secure servers hosted by the individual research groups and safeguarded by automated backup systems and/or backups to off-site servers maintained by their institution. We project that all of these systems will be in place for at least 10 years. All non-electronic data including detailed experimental procedures and observations are recorded in laboratory notebooks that do not leave the senior investigator's lab. Data should be accessible to the rest of the laboratory, but access is typically revoked when junior investigators leave the lab.
+Data will also be deposited into Northwestern Libraries’ institutional repository, Arch, upon publication. https://arch.library.northwestern.edu/ Arch assigns DOIs, making it easy to find the data. Necessary metadata and other resources to make the data accessible to future users will be submitted. Arch will preserve the data for future use. External investigators may choose to instead archive their data with similar repositories provided by the partner institution (such as Academic Commons at Columbia University, D-Scholarship@Pitt at the University of Pittsburgh, and Harvard University Archives).</t>
         </is>
       </c>
     </row>
@@ -1117,12 +1119,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Electronic files are stored on secure servers hosted by the individual research groups and safeguarded by automated backup systems and/or backups to off-site servers maintained by their institution. We project that all of these systems will be in place for at least 10 years. All non-electronic data including detailed experimental procedures and observations are recorded in laboratory notebooks that do not leave the senior investigator's lab. Data should be accessible to the rest of the laboratory, but access is typically revoked when junior investigators leave the lab.</t>
+          <t>Rationale. A discussion of the rationale or justification for the proposed data management plan including, for example, the potential impact of the data within the immediate field and in other fields, and any broader societal impact.</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1141,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Data will also be deposited into Northwestern Libraries’ institutional repository, Arch, upon publication. https://arch.library.northwestern.edu/ Arch assigns DOIs, making it easy to find the data. Necessary metadata and other resources to make the data accessible to future users will be submitted. Arch will preserve the data for future use. External investigators may choose to instead archive their data with similar repositories provided by the partner institution (such as Academic Commons at Columbia University, D-Scholarship@Pitt at the University of Pittsburgh, and Harvard University Archives).</t>
+          <t>The Department of Energy stipulates in their "Statement on Digital Data Management" that "To the greatest extent and with the fewest constraints possible, and consistent with the requirements and other principles of this Statement, data sharing should make digital research data available to and useful for the scientific community, industry, and the public." The Center will make every effort to comply with these guidelines. Data that is not deemed to be useful for a publication may still be archived at the discretion of the senior investigator overseeing the work, taking into the costs and benefits of doing so. The data acquired and preserved in the context of this proposal will be further governed by policies of the Northwestern University and its partner institutions pertaining to intellectual property, record retention, and data management.</t>
         </is>
       </c>
     </row>
@@ -1151,12 +1153,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Rationale. A discussion of the rationale or justification for the proposed data management plan including, for example, the potential impact of the data within the immediate field and in other fields, and any broader societal impact.</t>
+          <t>2. Data used in publications</t>
         </is>
       </c>
     </row>
@@ -1168,12 +1170,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>The Department of Energy stipulates in their "Statement on Digital Data Management" that "To the greatest extent and with the fewest constraints possible, and consistent with the requirements and other principles of this Statement, data sharing should make digital research data available to and useful for the scientific community, industry, and the public." The Center will make every effort to comply with these guidelines. Data that is not deemed to be useful for a publication may still be archived at the discretion of the senior investigator overseeing the work, taking into the costs and benefits of doing so. The data acquired and preserved in the context of this proposal will be further governed by policies of the Northwestern University and its partner institutions pertaining to intellectual property, record retention, and data management.</t>
+          <t>Data management plans should provide a plan for making all research data displayed in publications resulting from the proposed research open, machine-readable, and digitally accessible to the public at the time of publication. This includes data that are displayed in charts, figures, images, etc. In addition, the underlying digital research data used to generate the displayed data should be made as accessible as possible to the public in accordance with the Principles published in the DOE Policy for Digital Research Data Management. The published article should indicate how these data can be accessed.</t>
         </is>
       </c>
     </row>
@@ -1185,12 +1187,13 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2. Data used in publications</t>
+          <t>Research conducted within the Center will be published in appropriate scientific journals. The publisher may restrict the redistribution of that data. When not prohibitively expensive, open access will be selected. This will be supplemented by publishing the data in a preprint repository such as the arXiv subsequent to peer-reviewed publication if possible. All publishers we previously worked with allow arXiv publication or open access, so we do not anticipate a problem. Crystallographic data will be deposited into the ICSD or the CCDC databases for broad access. Data will also be disseminated through seminars at conferences and at other academic institutions. Raw data files can be provided to others upon request, but will be limited to their personal use only and cannot be redistributed without written consent from the PI.
+Access to data and results prior to publication or file for intellectual property is provided to all personnel involved in the project, after publication or filing for provisional patents, the data will be in the public domain and any further data will be provided to the community upon request or through appropriate websites (i.e. lab web sites). All of the fabrication methods, characterization results, and data acquired through the proposed research towards the development of the bioactive platforms will be shared with others through publication in conferences and journals.</t>
         </is>
       </c>
     </row>
@@ -1202,12 +1205,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Data management plans should provide a plan for making all research data displayed in publications resulting from the proposed research open, machine-readable, and digitally accessible to the public at the time of publication. This includes data that are displayed in charts, figures, images, etc. In addition, the underlying digital research data used to generate the displayed data should be made as accessible as possible to the public in accordance with the Principles published in the DOE Policy for Digital Research Data Management. The published article should indicate how these data can be accessed.</t>
+          <t>3. Data management resources</t>
         </is>
       </c>
     </row>
@@ -1219,12 +1222,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Research conducted within the Center will be published in appropriate scientific journals. The publisher may restrict the redistribution of that data. When not prohibitively expensive, open access will be selected. This will be supplemented by publishing the data in a preprint repository such as the arXiv subsequent to peer-reviewed publication if possible. All publishers we previously worked with allow arXiv publication or open access, so we do not anticipate a problem. Crystallographic data will be deposited into the ICSD or the CCDC databases for broad access. Data will also be disseminated through seminars at conferences and at other academic institutions. Raw data files can be provided to others upon request, but will be limited to their personal use only and cannot be redistributed without written consent from the PI.</t>
+          <t>Data management plans should consult and reference available information about data management resources to be used in the course of the proposed research. In particular, DMPs tht explicitly or implicitly commit data management resources at a facility beyond what is conventionally made available to approved users should be accompanied by written approval from that facility. In determining the resources available for data management at DOE Scientific User Facilities, researchers should consult the published description of data management resources and practices at that facility and reference it in the DMP. Information about other Office of Science facilities can be found in the additional guidance from the sponsporing program.</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1244,9 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Access to data and results prior to publication or file for intellectual property is provided to all personnel involved in the project, after publication or filing for provisional patents, the data will be in the public domain and any further data will be provided to the community upon request or through appropriate websites (i.e. lab web sites). All of the fabrication methods, characterization results, and data acquired through the proposed research towards the development of the bioactive platforms will be shared with others through publication in conferences and journals.</t>
+          <t>DMPs should consult and reference available information about data management resources to be used in the course of the proposed research. In particular, DMPs that explicitly or implicitly commit data management resources at a facility beyond what is conventionally made available to approved users should be accompanied by written approval from that facility. In determining the resources available for data management at Office of Science User Facilities, researchers should consult the published description of data management resources and practices at that facility and reference it in the DMP. Information about other Office of Science facilities can be found in the additional guidance from the sponsoring program.
+Data Repositories. Senior investigators typically archive relevant data using their own group servers. Whenever possible, investigators will be encouraged to also copy data to a centralized data server for CBES investigators. Additionally, researchers can archive data on repositories at their home institutions. For example, researchers at Northwestern are encouraged to deposit data into Northwestern Libraries’ institutional repository, Arch, upon publication (https://arch.library.northwestern.edu/). Arch assigns DOIs, making it easy to find the data. Necessary metadata and other resources to make the data accessible to future users will be submitted. Arch will preserve the data for future use.
+Data Volume. Generally, the volume of data generated by CBES researchers should not prohibit their deposition in available repositories. However, in cases where large volumes of data are generated (e.g., temperature/time dependent microscopy or X-ray studies), the data may need to be averaged, condensed, or minimally processed prior to deposition.</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1263,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>3. Data management resources</t>
+          <t>4. Confidentiality, security and rights</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1280,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Data management plans should consult and reference available information about data management resources to be used in the course of the proposed research. In particular, DMPs tht explicitly or implicitly commit data management resources at a facility beyond what is conventionally made available to approved users should be accompanied by written approval from that facility. In determining the resources available for data management at DOE Scientific User Facilities, researchers should consult the published description of data management resources and practices at that facility and reference it in the DMP. Information about other Office of Science facilities can be found in the additional guidance from the sponsporing program.</t>
+          <t>Data management plans must protect confidentiality, personal privacy, Personally Identifiable Information and U.S. national, homeland, and economic security; recognize proprietary interests, business confidential information, and intellectual property rights; avoid significant negative impact on innovation and U.S. competitiveness; and otherwise be consistent with all applicable laws, regulations, agreement terms and conditions, and DOE orders and policies. There is no requirement to share proprietary data.</t>
         </is>
       </c>
     </row>
@@ -1292,92 +1297,92 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DMPs should consult and reference available information about data management resources to be used in the course of the proposed research. In particular, DMPs that explicitly or implicitly commit data management resources at a facility beyond what is conventionally made available to approved users should be accompanied by written approval from that facility. In determining the resources available for data management at Office of Science User Facilities, researchers should consult the published description of data management resources and practices at that facility and reference it in the DMP. Information about other Office of Science facilities can be found in the additional guidance from the sponsoring program.</t>
+          <t>Data that may support intellectual property claims will be published only after we seek advice from the Northwestern Innovation and New Ventures Office (INVO). Such advice will be sought in a timely manner. The proposed research does not include the collection of any confidential personal information. The Director, the Executive Director for Research, and the Executive Committee will regularly review polices for data storage to ensure accessibility and security of CBES research data.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>sample2</t>
+          <t>sample3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Data Repositories. Senior investigators typically archive relevant data using their own group servers. Whenever possible, investigators will be encouraged to also copy data to a centralized data server for CBES investigators. Additionally, researchers can archive data on repositories at their home institutions. For example, researchers at Northwestern are encouraged to deposit data into Northwestern Libraries’ institutional repository, Arch, upon publication (https://arch.library.northwestern.edu/). Arch assigns DOIs, making it easy to find the data. Necessary metadata and other resources to make the data accessible to future users will be submitted. Arch will preserve the data for future use.</t>
+          <t>CPS 2015</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>sample2</t>
+          <t>sample3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Data Volume. Generally, the volume of data generated by CBES researchers should not prohibit their deposition in available repositories. However, in cases where large volumes of data are generated (e.g., temperature/time dependent microscopy or X-ray studies), the data may need to be averaged, condensed, or minimally processed prior to deposition.</t>
+          <t>Roles and responsibilities</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>sample2</t>
+          <t>sample3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>4. Confidentiality, security and rights</t>
+          <t>The Data Management Plan should clearly articulate how the PI and co-PIs plan to manage and disseminate data generated by the project. The plan should outline the rights and obligations of all parties as to their roles and responsibilities in the management and retention of research data, and consider changes that would occur should a PI or co-PI leave the institution or project. Any costs should be explained in the Budget Justification pages.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sample2</t>
+          <t>sample3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Data management plans must protect confidentiality, personal privacy, Personally Identifiable Information and U.S. national, homeland, and economic security; recognize proprietary interests, business confidential information, and intellectual property rights; avoid significant negative impact on innovation and U.S. competitiveness; and otherwise be consistent with all applicable laws, regulations, agreement terms and conditions, and DOE orders and policies. There is no requirement to share proprietary data.</t>
+          <t>Data will be generated at each of our institutional sites. The PI at each institution will be responsible for following the data management guidelines described below, and for saving the data to the RIC servers. This process of transferring all data to a central location will be facilitated by our research project coordinator. Our data management guidelines will be reviewed at the kickoff meeting for the project, and revisited briefly at each of our quarterly meetings with the PIs.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>sample2</t>
+          <t>sample3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Data that may support intellectual property claims will be published only after we seek advice from the Northwestern Innovation and New Ventures Office (INVO). Such advice will be sought in a timely manner. The proposed research does not include the collection of any confidential personal information. The Director, the Executive Director for Research, and the Executive Committee will regularly review polices for data storage to ensure accessibility and security of CBES research data.</t>
+          <t>Types of data</t>
         </is>
       </c>
     </row>
@@ -1389,12 +1394,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CPS 2015</t>
+          <t>The Data Management Plan should describe the types of data, samples, physical collections, software, curriculum materials, or other materials to be produced in the course of the project. It should then describe the expected types of data to be retained and shared, and the plans for doing so. The DMP should cover how data are to be managed and maintained during the project.</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1411,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Roles and responsibilities</t>
+          <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data. First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session. Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts. The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
         </is>
       </c>
     </row>
@@ -1423,12 +1428,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The Data Management Plan should clearly articulate how the PI and co-PIs plan to manage and disseminate data generated by the project. The plan should outline the rights and obligations of all parties as to their roles and responsibilities in the management and retention of research data, and consider changes that would occur should a PI or co-PI leave the institution or project. Any costs should be explained in the Budget Justification pages.</t>
+          <t>Policies for access and sharing and appropriate protection and privacy</t>
         </is>
       </c>
     </row>
@@ -1440,12 +1445,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Data will be generated at each of our institutional sites. The PI at each institution will be responsible for following the data management guidelines described below, and for saving the data to the RIC servers. This process of transferring all data to a central location will be facilitated by our research project coordinator. Our data management guidelines will be reviewed at the kickoff meeting for the project, and revisited briefly at each of our quarterly meetings with the PIs.</t>
+          <t>The Data Management Plan should describe the period of time the data will be retained and shared; factors that limit the ability to manage and share data, e.g., legal and ethical restrictions on access to human subjects data; and provisions for appropriate protection of privacy, confidentiality, security, and intellectual property.</t>
         </is>
       </c>
     </row>
@@ -1457,12 +1462,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Types of data</t>
+          <t>Data will be made available upon request, after the conclusion of each of study. The availability of data (raw and analyzed) will be advertised on the project’s website. Access will be free, but the original data collector/creator/principal investigator retains the right to use the data for analysis before making it publicly available. No patient identifying information will be included in any of the available data files. Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable. Experimental analyses results will be made available through peer-reviewed journal publications and conference presentations. The code needed to generate all published results will be documented clearly. Software generated under the project will be released under the GNU Public License, and available for free download on the labs’ websites. This includes code for each of our 3 experimental systems. We commit to speaking with any qualified scientist who wishes to discuss our results or the technology employed to obtain our results. There will be no copyright or licensing required for any of the data generated in this project. Research records will be archived for a minimum of seven years after final reporting or publication of a project. If any questions regarding the research, including but not limited to research integrity allegations, are raised during the seven- year retention period, the PI will keep the records until such questions are fully resolved.</t>
         </is>
       </c>
     </row>
@@ -1474,12 +1479,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The Data Management Plan should describe the types of data, samples, physical collections, software, curriculum materials, or other materials to be produced in the course of the project. It should then describe the expected types of data to be retained and shared, and the plans for doing so. The DMP should cover how data are to be managed and maintained during the project.</t>
+          <t>Data storage and preservation of access</t>
         </is>
       </c>
     </row>
@@ -1491,12 +1496,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data. First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session. Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts. The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
+          <t>The Data Management Plan should describe the mechanisms and formats for storing data and making them accessible to others, which may include third party facilities and repositories; and other types of information that would be maintained and shared regarding data, e.g. the means by which it was generated, detailed analytical and procedural information required to reproduce experimental results, and other metadata.</t>
         </is>
       </c>
     </row>
@@ -1508,12 +1513,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Policies for access and sharing and appropriate protection and privacy</t>
+          <t>The servers at the Rehabilitation Institute of Chicago will serve as the central repository for all collected data. Raw data files will be saved in either Matlab or comma-separated value (CSV) format. Code for converting between these formats will also be provided to ensure easy access. The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented. All raw data will be de-identified to ensure subject anonynimity. Upon request, data will be made available through the project's website, hosted on an archived server run by the RIC IT Team.</t>
         </is>
       </c>
     </row>
@@ -1525,131 +1530,133 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The Data Management Plan should describe the period of time the data will be retained and shared; factors that limit the ability to manage and share data, e.g., legal and ethical restrictions on access to human subjects data; and provisions for appropriate protection of privacy, confidentiality, security, and intellectual property.</t>
+          <t>Additional possible data management requirements</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>sample3</t>
+          <t>sample4</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Data will be made available upon request, after the conclusion of each of study. The availability of data (raw and analyzed) will be advertised on the project’s website. Access will be free, but the original data collector/creator/principal investigator retains the right to use the data for analysis before making it publicly available. No patient identifying information will be included in any of the available data files. Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable. Experimental analyses results will be made available through peer-reviewed journal publications and conference presentations. The code needed to generate all published results will be documented clearly. Software generated under the project will be released under the GNU Public License, and available for free download on the labs’ websites. This includes code for each of our 3 experimental systems. We commit to speaking with any qualified scientist who wishes to discuss our results or the technology employed to obtain our results. There will be no copyright or licensing required for any of the data generated in this project. Research records will be archived for a minimum of seven years after final reporting or publication of a project. If any questions regarding the research, including but not limited to research integrity allegations, are raised during the seven- year retention period, the PI will keep the records until such questions are fully resolved.</t>
+          <t>DATA MANAGEMENT PLAN</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>sample3</t>
+          <t>sample4</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Data storage and preservation of access</t>
+          <t>The P.I. has completed human subjects training. The research assistants will be required to complete human subjects training through the UCR Office of Research and Economic Development. The project will be submitted to the campus Institutional Review Board and requested revisions to the project based on feedback from the IRB will be incorporated prior to data collection. The researchers will ask all respondents to sign informed consent forms prior to interviews, as well as in connection with the collection of survey data. These consent forms will include information about how confidentiality of responses will be protected. The longevity analysis will collect data on the length of time clusters have operated (including the length of time between first hires and closures for those that have disbanded). We will collect data from a minimum of 36 institutions, attempting to find dates of operation for all clusters authorized at those institutions. The total number of clusters cannot be estimated at this time but is likely to encompass as many as 150-200. The comparative analysis will collect data on performance and attitudes from cluster participants. The performance data will include publications, citations, research grants, patents, licenses, and start-ups founded by members of interdisciplinary cluster hires, as well as those of a matched sample of faculty hired through normal departmental mechanisms. The survey data will include responses to five-page surveys from members of the interdisciplinary clusters. The P.I. will also collect interview data from cluster leads and university administrators. Performance and survey responses will be collected from a minimum of 72 individuals affiliated with interdisciplinary clusters (at least three individuals from four institutions each in six fields), and a matched sample of at least 72 individuals hired through normal departmental channels. Interview data will be collected from a minimum of 24 cluster leads and four administrators. If fields are drawn from multiple institutions, the number of interviews with cluster leads will reflect the number of institutions and the number of fields included in the sample. The number of interviews with university administrators will reflect the number of institutions included in the sample. The members of the project team will spot check coding on a 10 percent sample of individuals hired through cluster programs and a 10 percent sample of individual hired through normal departmental procedures. If problems arise in the validation of coding, more extensive checks will be conducted. Coders will be instructed on the requirements for producing high quality data, including meticulousness, conscientiousness, asking questions where uncertainties exist, and double checking work. Data will be backed up on a weekly basis on a hard drive kept in a locked cabinet in the project office. The data will be preserved exclusively on the two project computers and the back-up hard drive. Performance and survey data will be coded into STATA data files, including numeric institutional and cluster identifiers, for subsequent data analysis. Data collected from individual and institutions will be stripped of institutional identifications and given a letter title corresponding to the institution’s name. The University of California, Riverside, for example, might be labelled “Institution A.” Interviews will be tape recorded for consultation during the writing of papers and reports. To our knowledge, there will be little overlap between the data collected for this project and data collected by other researchers. The only project that may include overlapping data is that of Erin Leahey at the University of Arizona (SciSIP award #1461989). However, consultation with Prof. Leahey has led us to conclude that the amount of overlap is quite limited to the extent that it exists at all. Prof. Leahey’s work is focused on support for interdisciplinary activities on university campuses and includes evidence on university investments in interdisciplinary activities. In previous work, Prof. Leahey has collected data on publication rates and publication prominence of scholars working in interdisciplinary teams relative to scholars who are not working in such teams. We see little overlap in these data and the data the research team intends to collect. A robust study of interdisciplinary activity has been conducted at Stanford University by Prof. Daniel MacFarland. Although these data are relevant to our work, they are not exclusively or primarily focused on cluster hires. We do not intend to integrate either of these databases with the data we collect. All data will be coded and saved on password-protected computers in the project office. No data will be removed from the project office during the period of the project. The only individuals with access to the collected data will be the P.I. and research assistants. New research assistants will be advised of the essential care that must be taken with data collected for this project. Anyresearch assistants found to be handling data in a careless way will be immediately removed from the project staff. No names of individuals or institutions will be used in papers prepared by the project team without the explicit consent of the individuals and institutions. Data from the project will be preserved in data files stripped of individual and institutional names. These data files will include a small number of variables that will allow researchers to categorize the institutions. These variables include institutional size, Carnegie category, control (private, non-profit or public), and regional location. Following the completion of the project, the data archive will be made available on the project website to researchers who are interested in pursuing questions related to cluster hiring. The preservation format will be platform- independent. Following the end of the project, we will contact the Inter-University Consortium for Political and Social Research (ICPSR) at the University of Michigan about archiving the data on a permanent basis. We do not anticipate additional costs for preparing data and documentation for archiving. Potential secondary users of the data include institutional researchers, policy analysts, and higher education scholars. We do not intend to generate metadata from this project. We do not anticipate holding intellectual property rights to these data. The P.I., Professor Steven Brint, will be responsible for all data collection and precautions for the security and confidentiality of the data.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>sample3</t>
+          <t>sample5</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Data Management Plan should describe the mechanisms and formats for storing data and making them accessible to others, which may include third party facilities and repositories; and other types of information that would be maintained and shared regarding data, e.g. the means by which it was generated, detailed analytical and procedural information required to reproduce experimental results, and other metadata.</t>
+          <t>DATA MANAGEMENT PLAN</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>sample3</t>
+          <t>sample5</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>The servers at the Rehabilitation Institute of Chicago will serve as the central repository for all collected data. Raw data files will be saved in either Matlab or comma-separated value (CSV) format. Code for converting between these formats will also be provided to ensure easy access. The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented. All raw data will be de-identified to ensure subject anonynimity. Upon request, data will be made available through the project's website, hosted on an archived server run by the RIC IT Team.</t>
+          <t>REVIEW OF PROPOSAL COMPONENTS</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>sample3</t>
+          <t>sample5</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Additional possible data management requirements</t>
+          <t>The proposal is separated into three sections.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>sample4</t>
+          <t>sample5</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>question.text</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>DATA MANAGEMENT PLAN</t>
+          <t>Section 2.1 characterizes the aquifer formation that each groundwater well in the West taps and compares well construction patterns before and after the establishment of regulatory controls.
+Section 2.2 estimates groundwater components of the water budget (withdrawals and consumption) yearly (2016-2021) at the field scale.
+Section 2.3 integrates research and education through the Scientist Spotlight and Hydrologic Sciences Workshops.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>sample4</t>
+          <t>sample5</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>The P.I. has completed human subjects training. The research assistants will be required to complete human subjects training through the UCR Office of Research and Economic Development. The project will be submitted to the campus Institutional Review Board and requested revisions to the project based on feedback from the IRB will be incorporated prior to data collection. The researchers will ask all respondents to sign informed consent forms prior to interviews, as well as in connection with the collection of survey data. These consent forms will include information about how confidentiality of responses will be protected. The longevity analysis will collect data on the length of time clusters have operated (including the length of time between first hires and closures for those that have disbanded). We will collect data from a minimum of 36 institutions, attempting to find dates of operation for all clusters authorized at those institutions. The total number of clusters cannot be estimated at this time but is likely to encompass as many as 150-200. The comparative analysis will collect data on performance and attitudes from cluster participants. The performance data will include publications, citations, research grants, patents, licenses, and start-ups founded by members of interdisciplinary cluster hires, as well as those of a matched sample of faculty hired through normal departmental mechanisms. The survey data will include responses to five-page surveys from members of the interdisciplinary clusters. The P.I. will also collect interview data from cluster leads and university administrators. Performance and survey responses will be collected from a minimum of 72 individuals affiliated with interdisciplinary clusters (at least three individuals from four institutions each in six fields), and a matched sample of at least 72 individuals hired through normal departmental channels. Interview data will be collected from a minimum of 24 cluster leads and four administrators. If fields are drawn from multiple institutions, the number of interviews with cluster leads will reflect the number of institutions and the number of fields included in the sample. The number of interviews with university administrators will reflect the number of institutions included in the sample. The members of the project team will spot check coding on a 10 percent sample of individuals hired through cluster programs and a 10 percent sample of individual hired through normal departmental procedures. If problems arise in the validation of coding, more extensive checks will be conducted. Coders will be instructed on the requirements for producing high quality data, including meticulousness, conscientiousness, asking questions where uncertainties exist, and double checking work. Data will be backed up on a weekly basis on a hard drive kept in a locked cabinet in the project office. The data will be preserved exclusively on the two project computers and the back-up hard drive. Performance and survey data will be coded into STATA data files, including numeric institutional and cluster identifiers, for subsequent data analysis. Data collected from individual and institutions will be stripped of institutional identifications and given a letter title corresponding to the institution’s name. The University of California, Riverside, for example, might be labelled “Institution A.” Interviews will be tape recorded for consultation during the writing of papers and reports. To our knowledge, there will be little overlap between the data collected for this project and data collected by other researchers. The only project that may include overlapping data is that of Erin Leahey at the University of Arizona (SciSIP award #1461989). However, consultation with Prof. Leahey has led us to conclude that the amount of overlap is quite limited to the extent that it exists at all. Prof. Leahey’s work is focused on support for interdisciplinary activities on university campuses and includes evidence on university investments in interdisciplinary activities. In previous work, Prof. Leahey has collected data on publication rates and publication prominence of scholars working in interdisciplinary teams relative to scholars who are not working in such teams. We see little overlap in these data and the data the research team intends to collect. A robust study of interdisciplinary activity has been conducted at Stanford University by Prof. Daniel MacFarland. Although these data are relevant to our work, they are not exclusively or primarily focused on cluster hires. We do not intend to integrate either of these databases with the data we collect. All data will be coded and saved on password-protected computers in the project office. No data will be removed from the project office during the period of the project. The only individuals with access to the collected data will be the P.I. and research assistants. New research assistants will be advised of the essential care that must be taken with data collected for this project. Anyresearch assistants found to be handling data in a careless way will be immediately removed from the project staff. No names of individuals or institutions will be used in papers prepared by the project team without the explicit consent of the individuals and institutions. Data from the project will be preserved in data files stripped of individual and institutional names. These data files will include a small number of variables that will allow researchers to categorize the institutions. These variables include institutional size, Carnegie category, control (private, non-profit or public), and regional location. Following the completion of the project, the data archive will be made available on the project website to researchers who are interested in pursuing questions related to cluster hiring. The preservation format will be platform- independent. Following the end of the project, we will contact the Inter-University Consortium for Political and Social Research (ICPSR) at the University of Michigan about archiving the data on a permanent basis. We do not anticipate additional costs for preparing data and documentation for archiving. Potential secondary users of the data include institutional researchers, policy analysts, and higher education scholars. We do not intend to generate metadata from this project. We do not anticipate holding intellectual property rights to these data. The P.I., Professor Steven Brint, will be responsible for all data collection and precautions for the security and confidentiality of the data.</t>
+          <t>TYPES OF DATA</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1668,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>DATA MANAGEMENT PLAN</t>
+          <t>The PI and PhD student will be responsible for all data-related activities including: collection, documentation and metadata description, quality control, storage and backup, archiving, and sharing.</t>
         </is>
       </c>
     </row>
@@ -1678,12 +1685,14 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>REVIEW OF PROPOSAL COMPONENTS</t>
+          <t>The project will result in new sets of data, code, and tools. These outputs include: (a) source code to quality control, collate, and merge datasets, (b) open source models and budgets in R and/or python, and (c) sharable instructional materials (Scientist Spotlight activities and workshop materials).
+Input data: Available data will be systematically reviewed and downloaded. These data are likely available in the form of Microsoft Access files or Microsoft Excel spreadsheets; shapefiles or raster files; or text files or comma-delimited files. A multi-tier storage and quality assurance methodology will be adopted and will likely evolve as new datasets provide for challenging formats and organization.
+Produced Data: Datasets will be produced in Sections 2.1-2.3 of the proposal. These datasets will be formatted and shared in an open format (e.g., CSV) or in illustrator files (i.e., cross sections).</t>
         </is>
       </c>
     </row>
@@ -1695,12 +1704,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The proposal is separated into three sections.</t>
+          <t>DATA AND METADATA STANDARDS</t>
         </is>
       </c>
     </row>
@@ -1712,12 +1721,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Section 2.1 characterizes the aquifer formation that each groundwater well in the West taps and compares well construction patterns before and after the establishment of regulatory controls.</t>
+          <t>The data will be shared along with a README.txt, which will describe all files, their relationships, naming conventions, etc. Data elements and attributes will be described following ISO 19115 specifications and metadata schema and standards in Hydrology (e.g., following any establish standards of the Water Information Coordination Program’s Open Water Data Initiative (Larsen et al., 2016)) to allow for better interpretability and interoperability. Code and scripts produced in R and/or python will be documented for reproducibility purposes. The metadata for the codes will include: (1) description of the functions required to operate the analyses; (2) description of input parameters and outputs; and (3) test case, files and plots documenting the expected response of the model (Section 2.1) to a standard set of input parameters. Documentation will focus on the description of the functions, input parameters, outputs, the format of input data, instructions to run the model, and instructions to export the results. The outputs will be stored in CSV format with a metadata document describing the data structure of the output data.</t>
         </is>
       </c>
     </row>
@@ -1729,12 +1738,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Section 2.2 estimates groundwater components of the water budget (withdrawals and consumption) yearly (2016-2021) at the field scale.</t>
+          <t>POLICIES FOR ACCESS AND SHARING</t>
         </is>
       </c>
     </row>
@@ -1746,12 +1755,15 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Section 2.3 integrates research and education through the Scientist Spotlight and Hydrologic Sciences Workshops.</t>
+          <t>Raw data: Detailed information about how the data were obtained, including detailed contact information or websites for direct download and citations to all datasets will be provided to allow for accessibility and correct attribution to original collectors. All methodological procedures for data quality control and aggregation will be described in the data documentation. This information will be provided in the form of supplementary documentation for publications, in the README.txt file, and at the repository (record-level). All sharable raw data and the processed data will be archived in Dryad, https://datadryad.org, the agnostic open access repository backed by UCSB and the California Digital Library (CDL), which implements the latest best practices in data curation, publication, citation, and archival. Dryad assigns Digital Object Identifiers (DOIs) to deposited datasets and makes data discoverable through such services as the Thomson-Reuters Data Citation Index, Scopus, and Google Dataset Search. All data in Dryad is publicly accessible and released under a CC0 license. Data will be linked to publications and vice versa through DOIs.
+Scripts and code for analyses: All scripts and code will be archived in supplementary information appendices in publications as well as uploaded to Zenodo through the Dryad repository submission process along with the sharable raw and processed data in order to allow citations and a better connection to the research data curation and publication processes.
+Scientist spotlight: All scientist spotlight biographies, assignments, and open-access readings will be posted to an online Dashboard associated with the PI’s website, which is updated bi-monthly.
+Workshop frameworks: Workshop material will be shared with UCSB’s Diversity Committee through Google Drive; if workshop materials are fully supported by the Diversity Committee, these materials will also be shared through eSholarship for broader dissemination.</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1775,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>TYPES OF DATA</t>
+          <t>The PI is committed to publishing in open access journals. The UC is currently leading initiatives to assist faculty in paying for open access journals.</t>
         </is>
       </c>
     </row>
@@ -1780,12 +1792,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>The PI and PhD student will be responsible for all data-related activities including: collection, documentation and metadata description, quality control, storage and backup, archiving, and sharing.</t>
+          <t>POLICIES AND PROVISIONS FOR RE-USE, RE-DISTRIBUTION</t>
         </is>
       </c>
     </row>
@@ -1802,7 +1814,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The project will result in new sets of data, code, and tools. These outputs include: (a) source code to quality control, collate, and merge datasets, (b) open source models and budgets in R and/or python, and (c) sharable instructional materials (Scientist Spotlight activities and workshop materials).</t>
+          <t>All data deposited at Dryad will be publicly available under a CC0 license, meaning that others may freely build upon, enhance and reuse the works for any purposes without restriction under copyright or database law. CC0 does not exempt those who reuse the data from following community norms for scholarly communication, i.e., reusing the data in a way that is mindful of its limitations and citing the original data authors.</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1826,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Input data: Available data will be systematically reviewed and downloaded. These data are likely available in the form of Microsoft Access files or Microsoft Excel spreadsheets; shapefiles or raster files; or text files or comma-delimited files. A multi-tier storage and quality assurance methodology will be adopted and will likely evolve as new datasets provide for challenging formats and organization.</t>
+          <t>PLANS FOR ARCHIVING AND PRESERVATION OF ACCESS</t>
         </is>
       </c>
     </row>
@@ -1836,82 +1848,83 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Produced Data: Datasets will be produced in Sections 2.1-2.3 of the proposal. These datasets will be formatted and shared in an open format (e.g., CSV) or in illustrator files (i.e., cross sections).</t>
+          <t>UCSB Box will be used as the primary means to store and back up all collected input, generated output data sets and code, and educational materials over the course of the project and prior to data sharing. Box provides encryption of data at rest and in-transit, detailed logging of file actions, two-factor authentication, and access review of collaborators. Data will be accessed using Box Drive, which requires full disk encryption, firewall, and an antivirus software in order to install on a local computer. At the end of the project, all shareable data accompanied by the appropriate documentation, metadata, and code will be deposited into Dryad for long-term storage, preservation and accessibility. Deposits submitted to Dryad are curated prior to public release to conform with quality standards and enable future reuse.
+The source code for the research and education components (Sections 2.1, 2.2., and 2.3) will be saved, stored, and backed up on the UCSB Box. A copy of the code will also be submitted with each of the three planned publications. After the evaluation and refinement of the developed datasets and tools and once the research is completed and published, the final version of the tools and the documentation will be shared on the UCSB’s Dryad Data Repository. The final shareable instructional and teaching materials will also be shared via on a publicly accessible webpage (Scientist Spotlight ) and UCSB Google Drive(workshop materials) and Dryad in pdf format.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>DATA AND METADATA STANDARDS</t>
+          <t>Data Management Plan:</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The data will be shared along with a README.txt, which will describe all files, their relationships, naming conventions, etc. Data elements and attributes will be described following ISO 19115 specifications and metadata schema and standards in Hydrology (e.g., following any establish standards of the Water Information Coordination Program’s Open Water Data Initiative (Larsen et al., 2016)) to allow for better interpretability and interoperability. Code and scripts produced in R and/or python will be documented for reproducibility purposes. The metadata for the codes will include: (1) description of the functions required to operate the analyses; (2) description of input parameters and outputs; and (3) test case, files and plots documenting the expected response of the model (Section 2.1) to a standard set of input parameters. Documentation will focus on the description of the functions, input parameters, outputs, the format of input data, instructions to run the model, and instructions to export the results. The outputs will be stored in CSV format with a metadata document describing the data structure of the output data.</t>
+          <t>Types of data.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>POLICIES FOR ACCESS AND SHARING</t>
+          <t>The bulk of the data generated in this project will be 1, 2, 3, and 4 dimensional arrays of numbers and bytes representing fluid state variables generated via computer simulations of fluid flow. Images and video files will be created from the fluid data using both commercial packages, such as Matlab and free visualization packages such as VAPOR (developed at NCAR).</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Raw data: Detailed information about how the data were obtained, including detailed contact information or websites for direct download and citations to all datasets will be provided to allow for accessibility and correct attribution to original collectors. All methodological procedures for data quality control and aggregation will be described in the data documentation. This information will be provided in the form of supplementary documentation for publications, in the README.txt file, and at the repository (record-level). All sharable raw data and the processed data will be archived in Dryad, https://datadryad.org, the agnostic open access repository backed by UCSB and the California Digital Library (CDL), which implements the latest best practices in data curation, publication, citation, and archival. Dryad assigns Digital Object Identifiers (DOIs) to deposited datasets and makes data discoverable through such services as the Thomson-Reuters Data Citation Index, Scopus, and Google Dataset Search. All data in Dryad is publicly accessible and released under a CC0 license. Data will be linked to publications and vice versa through DOIs.</t>
+          <t>Data and metadata standards.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -1921,31 +1934,31 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Scripts and code for analyses: All scripts and code will be archived in supplementary information appendices in publications as well as uploaded to Zenodo through the Dryad repository submission process along with the sharable raw and processed data in order to allow citations and a better connection to the research data curation and publication processes.</t>
+          <t>The PI’s research group will adopt the longstanding practice that all generated data should be straightforwardly reproducible. Thus, codes are stored within the same directory on a mass storage system along with the data they generate. “Readme” files will also be provided for explanation of the directory content.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Scientist spotlight: All scientist spotlight biographies, assignments, and open-access readings will be posted to an online Dashboard associated with the PI’s website, which is updated bi-monthly.</t>
+          <t>Policies for access and sharing.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1955,99 +1968,99 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Workshop frameworks: Workshop material will be shared with UCSB’s Diversity Committee through Google Drive; if workshop materials are fully supported by the Diversity Committee, these materials will also be shared through eSholarship for broader dissemination.</t>
+          <t>Interested parties will be able to request data and codes at the end of the project. Such parties will be responsible for their own version control and execution.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The PI is committed to publishing in open access journals. The UC is currently leading initiatives to assist faculty in paying for open access journals.</t>
+          <t>Policies and provisions for re-use, re-distribution.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>POLICIES AND PROVISIONS FOR RE-USE, RE-DISTRIBUTION</t>
+          <t>Simulation data will in essence grow to several terrabytes with an associated cost of storage. Data will be made publicly available upon request at the end of the project. Although open-source, we envisage that intellectual rights to the code will be retained by the CU group. Dissemination of open-source software will be released once fully tested and published.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>All data deposited at Dryad will be publicly available under a CC0 license, meaning that others may freely build upon, enhance and reuse the works for any purposes without restriction under copyright or database law. CC0 does not exempt those who reuse the data from following community norms for scholarly communication, i.e., reusing the data in a way that is mindful of its limitations and citing the original data authors.</t>
+          <t>Plans for archiving and preservation of access.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample6</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>PLANS FOR ARCHIVING AND PRESERVATION OF ACCESS</t>
+          <t>Local data will be archived on the group’s mass storage system. As mentioned above, all data generated is archived with the entire code that generated it. Additionally, further backups of the data will be provided by CU’s NSF-funded research computing. We imagine the data being of relevance and stored for &gt; 10 years.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample7</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>UCSB Box will be used as the primary means to store and back up all collected input, generated output data sets and code, and educational materials over the course of the project and prior to data sharing. Box provides encryption of data at rest and in-transit, detailed logging of file actions, two-factor authentication, and access review of collaborators. Data will be accessed using Box Drive, which requires full disk encryption, firewall, and an antivirus software in order to install on a local computer. At the end of the project, all shareable data accompanied by the appropriate documentation, metadata, and code will be deposited into Dryad for long-term storage, preservation and accessibility. Deposits submitted to Dryad are curated prior to public release to conform with quality standards and enable future reuse.</t>
+          <t>Resource/Data Sharing Plan</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>sample5</t>
+          <t>sample7</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2057,14 +2070,14 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>The source code for the research and education components (Sections 2.1, 2.2., and 2.3) will be saved, stored, and backed up on the UCSB Box. A copy of the code will also be submitted with each of the three planned publications. After the evaluation and refinement of the developed datasets and tools and once the research is completed and published, the final version of the tools and the documentation will be shared on the UCSB’s Dryad Data Repository. The final shareable instructional and teaching materials will also be shared via on a publicly accessible webpage (Scientist Spotlight ) and UCSB Google Drive(workshop materials) and Dryad in pdf format.</t>
+          <t>The study investigators are committed to the open and timely dissemination of study data. The final datasets will include demographic and clinical assessment data obtained from interviews, questionnaires, and behavioral tasks collected from human subjects. The investigators will be fully compliant to the NIMH Data Archive (NDA) Data Sharing Terms and Conditions, including submitting and harmonizing all descriptive/raw data and analyzed data at the item and subject-level to the National Database for Clinical Trials (NDCT) according to the expected timeline (semi-annually, at the end of the grant or at the time of publication, whichever occurs first). The investigators will include appropriate language in participant consent documents to allow for the data sharing through NDA, and complete all required paperwork related to the submission and sharing. The investigators will certify the quality of all data prior to submission and review the data for accuracy after submission. The investigators will also associate the submitted data in NDA with the findings/publications (both positive and negative) using NDA-provided features. All submitted data will include an NDA Global Unique Identifier (GUID) and will not include personally identifiable information (PII). The exception to the above is the audio recordings of the treatment sessions. Even with the removal of all identifiers, we believe that it would be difficult if not impossible to protect the identities of participants given the voice characteristics of participants will be readily available and the relatively restricted area from which we are recruiting participants. Therefore, we are not planning to share this part of the data.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2074,14 +2087,14 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Data Management Plan:</t>
+          <t>Univ. of California, Riverside Data Management Plan</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2091,14 +2104,14 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Types of data.</t>
+          <t>1. Policy and Practice</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2108,14 +2121,14 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>The bulk of the data generated in this project will be 1, 2, 3, and 4 dimensional arrays of numbers and bytes representing fluid state variables generated via computer simulations of fluid flow. Images and video files will be created from the fluid data using both commercial packages, such as Matlab and free visualization packages such as VAPOR (developed at NCAR).</t>
+          <t>The Bourns College of Engineering (BCOE) at the University of California, Riverside , in partnership with the UCR Libraries and the California Digital Library, has established a new, custom data management system designed to make results of our research readily and reliably accessible. This system combines two services of the California Digital Library for the first time: an eScholarship series, a curated site where all BCOE investigators can store and disseminate their data, and EZID permanent identifiers for long-term identification and management of data resources. All principal investigators in BCOE are responsible for complying with sponsor policies regarding data management and accessibility. All have sufficient computing resources to store and process the data generated in their research. Every principal investigator has the ability to create his or her personal web site, and to make data sets available through that web site. Additionally, the eScholarship series (http://escholarship.org/uc/bcoe) provides a ready-made resource for dissemination. Researchers can submit materials to the eScholarship series site, where it is automatically given an EZID persistent identifier. All material on the site is indexed on Google, Scholar, and Melvyl/WorldCat. The California Digital Library also provides data backup services to avoid accidental loss of data. This partnership, which has resulted in the development of a new service that CDL can provide to other research organizations, makes our data widely available and searchable under the taxonomies, identifiers, and standards of universal data sharing systems envisioned for the near future (see Changing the Conduct of Science in the Information Age , NSF, June 2011).</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2125,14 +2138,14 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Data and metadata standards.</t>
+          <t>2. Scope</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2142,14 +2155,14 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>The PI’s research group will adopt the longstanding practice that all generated data should be straightforwardly reproducible. Thus, codes are stored within the same directory on a mass storage system along with the data they generate. “Readme” files will also be provided for explanation of the directory content.</t>
+          <t>This Data Management Plan addresses the NSF policy that primary data “commonly accepted in the scientific community as necessary to validate research findings” be made available at little or no cost to the PI or project. In accordance with this policy and guidance from the Office of Management and Budget, this plan does not include preliminary analyses (including raw data), drafts of scientific papers, plans for future research, peer reviews, or communications with colleagues. Data that must be withheld long enough to enable peer review and publication/dissemination or protection of intellectual property is subject to this plan only after those steps have taken place. Data will be available for access and sharing as soon as is reasonably possible, and no later than two years after its acquisition. The data will be preserved for at least three years beyond the award period, as required by NSF guidelines. The release of data about students or any other human subjects is subject to policies and restrictions in protocols adopted by the relevant Institutional Research Board (IRB) and the Family Educational Rights and Privacy Act (FERPA) regulations. The proposed project will develop programming, compiler, and runtime support for applications, as described in this proposal. The implementations will be made available to other researchers. All code will be preserved and maintained for a minimum of three years beyond the award period as required by NSF guidelines. In addition, sample adaptive versions of applications that will be developed in this work will also be made available.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2159,14 +2172,14 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Policies for access and sharing.</t>
+          <t>3. Data and Metadata Format and Content</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2176,14 +2189,14 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Interested parties will be able to request data and codes at the end of the project. Such parties will be responsible for their own version control and execution.</t>
+          <t>The software will be made available in source code form and so will the applications developed. This will allow other researchers to so not only use it but also modify it for their use. All materials uploaded to the eScholarship site from UCR will be tagged uniformly with metadata about the source and nature of the data. Any electronic file format (e.g., text, spreadsheets, images) can be accepted. As a service to assure that materials are formatted correctly, a curator from the College reviews all submissions before they are accepted.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2193,14 +2206,14 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Policies and provisions for re-use, re-distribution.</t>
+          <t>4. Accessibility and Data Protection</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2210,14 +2223,14 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Simulation data will in essence grow to several terrabytes with an associated cost of storage. Data will be made publicly available upon request at the end of the project. Although open-source, we envisage that intellectual rights to the code will be retained by the CU group. Dissemination of open-source software will be released once fully tested and published.</t>
+          <t>Materials will be searchable through a number of databases and search engines, including Google and Google Scholar. As noted in Section 2 (Scope), data will be made available only after appropriate steps have been taken to protect intellectual property. Confidential material will be handled according to policies and protocols for human subjects, FERPA, and any other applicable regulations and restrictions. Stored materials are downloadable but not editable, and they are backed up to assure no loss of data. All uploads are approved by a curator before they are published.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2227,14 +2240,14 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Plans for archiving and preservation of access.</t>
+          <t>5. Derivative Products</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>sample6</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2244,31 +2257,31 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Local data will be archived on the group’s mass storage system. As mentioned above, all data generated is archived with the entire code that generated it. Additionally, further backups of the data will be provided by CU’s NSF-funded research computing. We imagine the data being of relevance and stored for &gt; 10 years.</t>
+          <t>All materials will contain acknowledgement of NSF support as per NSF policy: “ This material is based upon work supported by the National Science Foundation under Grant No. (NSF grant number). ” Additionally, materials will contain a disclaimer that “ any opinions, findings, and conclusions or recommendations expressed in this material are those of the author(s) and do not necessarily reflect the views of the National Science Foundation .” In keeping with standard ethical practices, it is expected that subsequent users of the data will acknowledge the source.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>sample7</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Resource/Data Sharing Plan</t>
+          <t>6. Archiving and Access</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>sample7</t>
+          <t>sample8</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2278,14 +2291,14 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>The study investigators are committed to the open and timely dissemination of study data. The final datasets will include demographic and clinical assessment data obtained from interviews, questionnaires, and behavioral tasks collected from human subjects. The investigators will be fully compliant to the NIMH Data Archive (NDA) Data Sharing Terms and Conditions, including submitting and harmonizing all descriptive/raw data and analyzed data at the item and subject-level to the National Database for Clinical Trials (NDCT) according to the expected timeline (semi-annually, at the end of the grant or at the time of publication, whichever occurs first). The investigators will include appropriate language in participant consent documents to allow for the data sharing through NDA, and complete all required paperwork related to the submission and sharing. The investigators will certify the quality of all data prior to submission and review the data for accuracy after submission. The investigators will also associate the submitted data in NDA with the findings/publications (both positive and negative) using NDA-provided features. All submitted data will include an NDA Global Unique Identifier (GUID) and will not include personally identifiable information (PII). The exception to the above is the audio recordings of the treatment sessions. Even with the removal of all identifiers, we believe that it would be difficult if not impossible to protect the identities of participants given the voice characteristics of participants will be readily available and the relatively restricted area from which we are recruiting participants. Therefore, we are not planning to share this part of the data.</t>
+          <t>If the PI leaves UCR, the products in the eScholarship series will remain stored there. PI is free to reproduce and repost these materials at his/her new institution.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2295,14 +2308,14 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Univ. of California, Riverside Data Management Plan</t>
+          <t>CAREER: HIGH-RESOLUTION NMR FOR PARAMAGNETIC SODIUM ELECTRODES</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2312,14 +2325,14 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>1. Policy and Practice</t>
+          <t>Products of Research</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2329,14 +2342,14 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>The Bourns College of Engineering (BCOE) at the University of California, Riverside , in partnership with the UCR Libraries and the California Digital Library, has established a new, custom data management system designed to make results of our research readily and reliably accessible. This system combines two services of the California Digital Library for the first time: an eScholarship series, a curated site where all BCOE investigators can store and disseminate their data, and EZID permanent identifiers for long-term identification and management of data resources. All principal investigators in BCOE are responsible for complying with sponsor policies regarding data management and accessibility. All have sufficient computing resources to store and process the data generated in their research. Every principal investigator has the ability to create his or her personal web site, and to make data sets available through that web site. Additionally, the eScholarship series (http://escholarship.org/uc/bcoe) provides a ready-made resource for dissemination. Researchers can submit materials to the eScholarship series site, where it is automatically given an EZID persistent identifier. All material on the site is indexed on Google, Scholar, and Melvyl/WorldCat. The California Digital Library also provides data backup services to avoid accidental loss of data. This partnership, which has resulted in the development of a new service that CDL can provide to other research organizations, makes our data widely available and searchable under the taxonomies, identifiers, and standards of universal data sharing systems envisioned for the near future (see Changing the Conduct of Science in the Information Age , NSF, June 2011).</t>
+          <t>Battery material samples will be synthesized in powder form and identified through a consistent and systematic labeling procedure, which will include sample composition, name of researcher and date. Experimental data generated over the course of the research will include synthesis procedures and results from characterization of battery electrode samples. Digital characterization data in tabular form will be produced by electrochemical testing, X-ray diffraction, solid-state NMR spectroscopy, EPR spectroscopy, magnetometry, impedance spectroscopy, X-ray photoelectron and absorption spectroscopy, and Mössbauer spectroscopy measurements. Rietveld refinements of scattering data will generate crystallographic data. Scanning electron microscopy will generate images. Synthetic work and optimization of NMR experimental procedures will be documented in lab notebooks and generate physical data. The Van der Ven group’s CASM software will be extended to enable the simulation of finite temperature NMR spectra of paramagnetic materials. First principles and Monte Carlo simulations will produce text files, density of states plots and two-dimensional charge density maps. Educational and outreach materials, and assessment results, will be digitized.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2346,14 +2359,14 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2. Scope</t>
+          <t>Data Format Standards</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2363,14 +2376,14 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>This Data Management Plan addresses the NSF policy that primary data “commonly accepted in the scientific community as necessary to validate research findings” be made available at little or no cost to the PI or project. In accordance with this policy and guidance from the Office of Management and Budget, this plan does not include preliminary analyses (including raw data), drafts of scientific papers, plans for future research, peer reviews, or communications with colleagues. Data that must be withheld long enough to enable peer review and publication/dissemination or protection of intellectual property is subject to this plan only after those steps have taken place. Data will be available for access and sharing as soon as is reasonably possible, and no later than two years after its acquisition. The data will be preserved for at least three years beyond the award period, as required by NSF guidelines. The release of data about students or any other human subjects is subject to policies and restrictions in protocols adopted by the relevant Institutional Research Board (IRB) and the Family Educational Rights and Privacy Act (FERPA) regulations. The proposed project will develop programming, compiler, and runtime support for applications, as described in this proposal. The implementations will be made available to other researchers. All code will be preserved and maintained for a minimum of three years beyond the award period as required by NSF guidelines. In addition, sample adaptive versions of applications that will be developed in this work will also be made available.</t>
+          <t>In order to allow for interoperability, reproducibility, and reuse, all data will be stored and saved in standard and open formats. Experimental characterization data will be stored and saved as, e.g., ASCII, CSV, Word, Matlab and Python files. Microscope images will be stored as portable graphic files (.tif, .jpg or .png format). Crystallographic data will be reported in standard crystallographic information framework (*.cif) format to facilitate visualization and further analysis through widely available software tools (VESTA, cif2file, etc.). Crystallographic data for previously-unreported compounds/structures will be uploaded to the ICSD database. First principles simulation input and output files (generated with the VASP and CRYSTAL codes) will be stored as rich text format (*.rtf) files for readability across many programs and platforms. The CRYSTAL code manual will be provided along CRYSTAL input/output data to allow for interpretation of variables. Both CRYSTAL and VASP manuals are also available online. The Van der Ven group's CASM software currently interfaces with VASP, automates the construction of effective Hamiltonians and subjects them to Monte Carlo simulations. CASM organizes all the files associated with VASP calculations into a standard structure that can be accessed by subsequent runs of CASM, either by the same user or by a new user. A similar CASM interface and infrastructure will be developed here for CRYSTAL calculations of NMR properties. The uniform file structure enforced by CASM for the effective Hamiltonian construction and the large number of Monte Carlo simulations that are necessary to construct, e.g., temperature composition phase diagrams, will be extended to include Fermi contact shifts and electric field gradient tensors. This will ensure that results from calculations performed by different users are in a format that is readily accessible, either by CASM or directly by different people.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -2380,14 +2393,14 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>3. Data and Metadata Format and Content</t>
+          <t>Access and sharing</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -2397,14 +2410,14 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>The software will be made available in source code form and so will the applications developed. This will allow other researchers to so not only use it but also modify it for their use. All materials uploaded to the eScholarship site from UCR will be tagged uniformly with metadata about the source and nature of the data. Any electronic file format (e.g., text, spreadsheets, images) can be accepted. As a service to assure that materials are formatted correctly, a curator from the College reviews all submissions before they are accepted.</t>
+          <t>The Program Toolkit and Activity Plans developed for the educational and outreach activities in partnership with Jamboree Housing (JH) will be uploaded to JH’s filesharing system for broad and free dissemination to their different centers and partners in California. All of the research results will be disseminated through peer-reviewed publications, conference presentations, and annual reports. The supporting information accompanying publications will include detailed experimental/simulation/synthetic procedures, as well as detailed information on models used for data analysis. All of the journals of interest to the group make supporting information files publicly-available online free of charge. In addition, all publication pre-prints will be made freely available, along with supplementary information, on the UC eScholarship website. Over the course of the project, digital data will be internally stored and shared for collaborative work on the UCSB-administered, Box platform with unlimited cloud storage. The privacy, security and intellectual property protection of data stored in this manner are guaranteed by the privacy policy and terms of service contract between University of California and Box. As a means of making data accessible and searchable, data collected over the course of this project will be stored in the data repository Dryad. enables easy data upload and description, and creates digital object identifiers (DOIs) for each dataset to help manage long-term data sharing through digital organization. We note that CASM systematically organizes all first-principles calculations that have been performed on a given system and has tools to query a wide range of properties for each calculation. Furthermore, any structure with a chemical ordering, magnetic ordering or a structural distortion that has been made "by hand" can be imported in a CASM project and made to be consistent with the automatically enumerated configurations. Hence, for each system of interest to this work, a structured CASM results packet that can easily be queried will be created (consisting of the results of electronic structure calculations, effective Hamiltonian interaction parameters and basis functions and Monte Carlo results) and uploaded to Dryad. is free of charge for UCSB researchers and can be accessed using a personal ORCID. CASM is an open source software package released under the GNU Lesser General Public License (LGPL) and available free of charge via the prisms-center conda channel at https://anaconda.org/prisms-center. All additions of the CASM software developed during this project will be incorporated into the CASM software and made accessible free of charge and open source under a similar LGPL license. Demonstrations on how to access and use CASM’s NMR extensions (and conditions under which they can use and modify the code) will be uploaded to the CASM software website: https://prisms-center.github.io/CASMcode_docs/.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -2414,14 +2427,14 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>4. Accessibility and Data Protection</t>
+          <t>Policies and provisions for re-use, re-distribution, and production of derivatives</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -2431,14 +2444,14 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Materials will be searchable through a number of databases and search engines, including Google and Google Scholar. As noted in Section 2 (Scope), data will be made available only after appropriate steps have been taken to protect intellectual property. Confidential material will be handled according to policies and protocols for human subjects, FERPA, and any other applicable regulations and restrictions. Stored materials are downloadable but not editable, and they are backed up to assure no loss of data. All uploads are approved by a curator before they are published.</t>
+          <t>All data will be stored in Dryad and will be available under a public domain, creative commons license (CC0). Note that while a personal ORCID is needed to deposit data in Dryad, no ORCID is required to search, find and download datasets. The existing open source software infrastructure within CASM that serves as a foundation to this project, is already licensed by the Regents of the University of California under the "LGPL" open source license, and distributed via the prisms-center conda channel, permitting non-exclusive use of the software. Additions to CASM will be released as LGPL to follow the current licensing of CASM.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2448,14 +2461,14 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>5. Derivative Products</t>
+          <t>Archiving of Data, Samples, and Other Relevant Research Products</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample9</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -2465,65 +2478,65 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>All materials will contain acknowledgement of NSF support as per NSF policy: “ This material is based upon work supported by the National Science Foundation under Grant No. (NSF grant number). ” Additionally, materials will contain a disclaimer that “ any opinions, findings, and conclusions or recommendations expressed in this material are those of the author(s) and do not necessarily reflect the views of the National Science Foundation .” In keeping with standard ethical practices, it is expected that subsequent users of the data will acknowledge the source.</t>
+          <t>Laboratory notebooks and samples will be retained for a minimum of 5 years following the conclusion of the program and will remain the property of UC Santa Barbara and kept on campus after students graduate. All digital data produced over the course of the project and stored on Box will be moved to Dryad after completion of the project for indefinite storage (&gt;5 years).</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>6. Archiving and Access</t>
+          <t>DATA MANAGEMENT</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>sample8</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>If the PI leaves UCR, the products in the eScholarship series will remain stored there. PI is free to reproduce and repost these materials at his/her new institution.</t>
+          <t>1. Policy and Practice</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>CAREER: HIGH-RESOLUTION NMR FOR PARAMAGNETIC SODIUM ELECTRODES</t>
+          <t>We will ensure that the data obtained and this study will be made available to the research community. The Bourns College of Engineering (BCOE) at UCR, in partnership with the UCR Libraries and the California Digital Library, has established a new, custom data management system designed to make results of our research readily and reliably accessible. This system combines two services of the California Digital Library (CDL) for the first time: an eScholarship series, a curated site where all BCOE investigators can store and disseminate their data, and EZID permanent identifiers for long-term identification and management of data resources. All principal investigators in BCOE are responsible for complying with sponsor policies regarding data management and accessibility. All have sufficient computing resources to store and process the data generated in their research. Every principal investigator has the ability to create his or her personal web site, and to make data sets available through that web site. Additionally, the eScholarship series (http:/escholarship.org/uc/search?entity=bcoe) provides another venue for dissemination. Researchers can submit materials to the eScholarship series site, where it is automatically given an EZID persistent identifier. All material on the site is indexed on Google, Scholar, and Melvyl/WorldCat. CDL also provides data backup services to avoid accidental loss of data. This partnership, which has resulted in the development of a new service that CDL can provide to other research organizations, makes our data widely available and searchable under the taxonomies, identifiers, and standards of universal data sharing systems envisioned for the near future (see Changing the Conduct of Science in the Information Age , NSF, June 2011).</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -2533,14 +2546,14 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Products of Research</t>
+          <t>2. Scope</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2550,14 +2563,14 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Battery material samples will be synthesized in powder form and identified through a consistent and systematic labeling procedure, which will include sample composition, name of researcher and date. Experimental data generated over the course of the research will include synthesis procedures and results from characterization of battery electrode samples. Digital characterization data in tabular form will be produced by electrochemical testing, X-ray diffraction, solid-state NMR spectroscopy, EPR spectroscopy, magnetometry, impedance spectroscopy, X-ray photoelectron and absorption spectroscopy, and Mössbauer spectroscopy measurements. Rietveld refinements of scattering data will generate crystallographic data. Scanning electron microscopy will generate images. Synthetic work and optimization of NMR experimental procedures will be documented in lab notebooks and generate physical data. The Van der Ven group’s CASM software will be extended to enable the simulation of finite temperature NMR spectra of paramagnetic materials. First principles and Monte Carlo simulations will produce text files, density of states plots and two-dimensional charge density maps. Educational and outreach materials, and assessment results, will be digitized.</t>
+          <t>This Data Management Plan addresses the NSF policy that primary data “commonly accepted in the scientific community as necessary to validate research findings” be made available at little or no cost to the PI or project. In accordance with this policy and guidance from the Office of Management and Budget, this plan does not include preliminary analyses (including raw data), drafts of scientific papers, plans for future research, peer reviews, or communications with colleagues. Data that must be withheld long enough to enable peer review and publication/dissemination or protection of intellectual property is subject to this plan only after those steps have taken place. Under this application, we will determine the effectiveness the proposed nano-vesicles (NETs) as photo-theranostic materials for fluorescence imaging and photothermal therapies. The release of data about students or any other human subjects is subject to policies and restrictions in protocols adopted by the relevant Institutional Research Board (IRB) and the Family Educational Rights and Privacy Act (FERPA) regulations.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -2567,14 +2580,14 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Data Format Standards</t>
+          <t>3. Data and Metadata Format and Contents</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -2584,14 +2597,14 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>In order to allow for interoperability, reproducibility, and reuse, all data will be stored and saved in standard and open formats. Experimental characterization data will be stored and saved as, e.g., ASCII, CSV, Word, Matlab and Python files. Microscope images will be stored as portable graphic files (.tif, .jpg or .png format). Crystallographic data will be reported in standard crystallographic information framework (*.cif) format to facilitate visualization and further analysis through widely available software tools (VESTA, cif2file, etc.). Crystallographic data for previously-unreported compounds/structures will be uploaded to the ICSD database. First principles simulation input and output files (generated with the VASP and CRYSTAL codes) will be stored as rich text format (*.rtf) files for readability across many programs and platforms. The CRYSTAL code manual will be provided along CRYSTAL input/output data to allow for interpretation of variables. Both CRYSTAL and VASP manuals are also available online. The Van der Ven group's CASM software currently interfaces with VASP, automates the construction of effective Hamiltonians and subjects them to Monte Carlo simulations. CASM organizes all the files associated with VASP calculations into a standard structure that can be accessed by subsequent runs of CASM, either by the same user or by a new user. A similar CASM interface and infrastructure will be developed here for CRYSTAL calculations of NMR properties. The uniform file structure enforced by CASM for the effective Hamiltonian construction and the large number of Monte Carlo simulations that are necessary to construct, e.g., temperature composition phase diagrams, will be extended to include Fermi contact shifts and electric field gradient tensors. This will ensure that results from calculations performed by different users are in a format that is readily accessible, either by CASM or directly by different people.</t>
+          <t>We will make the proposed nano-vesicles (NETs) available to interested investigators who would like to use them in their scientific research. We will publish our results, and present them results in relevant conferences, workshops, seminars, and teaching forums. Additionally, we will provide our results to any national resources and or databases on nanoparticles that compile and maintain such information. As an example, we will contribute to the nanotechnology information library (NIL) (http://nanoparticlelibrary.net/index.asp), which is maintained by the National Institute for Occupational Safety and Health (NIOSH). Data that must be withheld long enough to enable peer review and publication/dissemination or protection of intellectual property will be subject after appropriate steps have taken place. Confidential material will be handled according to policies and protocols at UCR, Family Educational Rights and Privacy Act (FERPA), and any other applicable regulations and restrictions. All materials uploaded to the eScholarship site will be tagged uniformly with metadata about the source and nature of the data. Any electronic file format (e.g., text, spreadsheets, images) can be accepted. As a service to assure that materials are formatted correctly, a curator from the College reviews all submissions before they are accepted.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -2601,14 +2614,14 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Access and sharing</t>
+          <t>4. Accessibility and Data Protection</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -2618,14 +2631,14 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>The Program Toolkit and Activity Plans developed for the educational and outreach activities in partnership with Jamboree Housing (JH) will be uploaded to JH’s filesharing system for broad and free dissemination to their different centers and partners in California. All of the research results will be disseminated through peer-reviewed publications, conference presentations, and annual reports. The supporting information accompanying publications will include detailed experimental/simulation/synthetic procedures, as well as detailed information on models used for data analysis. All of the journals of interest to the group make supporting information files publicly-available online free of charge. In addition, all publication pre-prints will be made freely available, along with supplementary information, on the UC eScholarship website. Over the course of the project, digital data will be internally stored and shared for collaborative work on the UCSB-administered, Box platform with unlimited cloud storage. The privacy, security and intellectual property protection of data stored in this manner are guaranteed by the privacy policy and terms of service contract between University of California and Box. As a means of making data accessible and searchable, data collected over the course of this project will be stored in the data repository Dryad. enables easy data upload and description, and creates digital object identifiers (DOIs) for each dataset to help manage long-term data sharing through digital organization. We note that CASM systematically organizes all first-principles calculations that have been performed on a given system and has tools to query a wide range of properties for each calculation. Furthermore, any structure with a chemical ordering, magnetic ordering or a structural distortion that has been made "by hand" can be imported in a CASM project and made to be consistent with the automatically enumerated configurations. Hence, for each system of interest to this work, a structured CASM results packet that can easily be queried will be created (consisting of the results of electronic structure calculations, effective Hamiltonian interaction parameters and basis functions and Monte Carlo results) and uploaded to Dryad. is free of charge for UCSB researchers and can be accessed using a personal ORCID. CASM is an open source software package released under the GNU Lesser General Public License (LGPL) and available free of charge via the prisms-center conda channel at https://anaconda.org/prisms-center. All additions of the CASM software developed during this project will be incorporated into the CASM software and made accessible free of charge and open source under a similar LGPL license. Demonstrations on how to access and use CASM’s NMR extensions (and conditions under which they can use and modify the code) will be uploaded to the CASM software website: https://prisms-center.github.io/CASMcode_docs/.</t>
+          <t>Materials will be searchable through a number of databases and search engines, including Google and Google Scholar. As noted in Section 2 (Scope), data will be made available only after appropriate steps have been taken to protect intellectual property. Confidential material will be handled according to policies and protocols for human subjects, FERPA, and any other applicable regulations and restrictions. Stored materials are downloadable but not editable, and they are backed up to assure no loss of data. All uploads are approved by a curator before they are published.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -2635,14 +2648,14 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Policies and provisions for re-use, re-distribution, and production of derivatives</t>
+          <t>5. Derivative Products</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -2652,14 +2665,14 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>All data will be stored in Dryad and will be available under a public domain, creative commons license (CC0). Note that while a personal ORCID is needed to deposit data in Dryad, no ORCID is required to search, find and download datasets. The existing open source software infrastructure within CASM that serves as a foundation to this project, is already licensed by the Regents of the University of California under the "LGPL" open source license, and distributed via the prisms-center conda channel, permitting non-exclusive use of the software. Additions to CASM will be released as LGPL to follow the current licensing of CASM.</t>
+          <t>All materials will contain acknowledgement of NSF support as per NSF policy: “ This material is based upon work supported by the National Science Foundation under Grant No. (NSF grant number). ” Additionally, materials will contain a disclaimer that “ any opinions, findings, and conclusions or recommendations expressed in this material are those of the author(s) and do not necessarily reflect the views of the National Science Foundation .” In keeping with standard ethical practices, it is expected that subsequent users of the data will acknowledge the source.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -2669,14 +2682,14 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Archiving of Data, Samples, and Other Relevant Research Products</t>
+          <t>6. Archiving and Access</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>sample9</t>
+          <t>sample10</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -2686,48 +2699,48 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Laboratory notebooks and samples will be retained for a minimum of 5 years following the conclusion of the program and will remain the property of UC Santa Barbara and kept on campus after students graduate. All digital data produced over the course of the project and stored on Box will be moved to Dryad after completion of the project for indefinite storage (&gt;5 years).</t>
+          <t>It is understood that the NSF Engineering Directorate requires data to be made available for a minimum of three years after conclusion of the award or public release, whichever is later. If the PI leaves his institution, the products will remain stored in relevant databases. PI is free to reproduce and repost these materials at new institution.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample11</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>DATA MANAGEMENT</t>
+          <t>3.3.3 Data Management Plan</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample11</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>1. Policy and Practice</t>
+          <t>All participants in the proposed project with access to the numerical codes and computational data will conform closely to NASA policy on preserving and sharing of the research data and gathered in the course of the proposed project. The data acquired and preserved in the context of this proposal will be further governed by UCSB’s policies pertaining to intellectual property, record retention, and data management.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample11</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -2737,218 +2750,224 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>We will ensure that the data obtained and this study will be made available to the research community. The Bourns College of Engineering (BCOE) at UCR, in partnership with the UCR Libraries and the California Digital Library, has established a new, custom data management system designed to make results of our research readily and reliably accessible. This system combines two services of the California Digital Library (CDL) for the first time: an eScholarship series, a curated site where all BCOE investigators can store and disseminate their data, and EZID permanent identifiers for long-term identification and management of data resources. All principal investigators in BCOE are responsible for complying with sponsor policies regarding data management and accessibility. All have sufficient computing resources to store and process the data generated in their research. Every principal investigator has the ability to create his or her personal web site, and to make data sets available through that web site. Additionally, the eScholarship series (http:/escholarship.org/uc/search?entity=bcoe) provides another venue for dissemination. Researchers can submit materials to the eScholarship series site, where it is automatically given an EZID persistent identifier. All material on the site is indexed on Google, Scholar, and Melvyl/WorldCat. CDL also provides data backup services to avoid accidental loss of data. This partnership, which has resulted in the development of a new service that CDL can provide to other research organizations, makes our data widely available and searchable under the taxonomies, identifiers, and standards of universal data sharing systems envisioned for the near future (see Changing the Conduct of Science in the Information Age , NSF, June 2011).</t>
+          <t>Digital products from this project include: 1) a numerical code that can predict the ADR performance of a magnetic refrigerant based on DFT and DFPT simulation of magnon and phonon properties. The computer code will be published on the open-source website GitHub. PI Liao has published homemade code on GitHub before (https://github.com/nanoengineering/EPW-nano). 2) a numerical code that solves the coupled magnon-phonon Boltzmann transport equations. This software will be written in Python and published and regularly maintained/updated on the open-source website GitHub. 3) Data from first-principles simulations, including magnon and phonon transport properties of selected magnetic materials. Metadata that describes simulation conditions will also be generated, indexed, and archived together with the raw data. Raw simulation data will be carefully curated and archived. The team will archive all data in local computers and a centralized data storage system based on external hard drives, which is synchronized to cloud storage (UCSB provides unlimited Google Drive storage space to researchers). Graduate students participating in this project will be directly responsible for collecting, curating, and archiving the data. They will be trained by PI Liao before the start of the project on the proper protocol of handling data. The stored data will be periodically (at least monthly) inspected by PI Liao. In the event of the departure of key personnel, a written document detailing the content and the condition of the data that they are responsible for should be prepared and data transfer and training should be conducted before the departure.
+We will publish primary results expeditiously in peer-reviewed journals, supported by relevant data in the supplementary documents along with the published papers. Raw data supporting published papers will be made available to the public automatically by depositing the data to the open-access repository Figshare, and the web link will be provided in the published paper. The raw data will be properly annotated and detailed metadata that describes the content, format, organization of the raw data will also be provided to help interpret the raw data. If processed data is used in the publication, the processing procedure will be described in detail in the paper. We will provide full assistance in terms of raw data availability, data processing software and error analysis for other researchers to validate and reproduce our results. We will make peer-reviewed publications from this project all available to the public by depositing the accepted manuscripts to depositories like arXiv and PubMed Central.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2. Scope</t>
+          <t>C-GEM: Plan for Data Management</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>This Data Management Plan addresses the NSF policy that primary data “commonly accepted in the scientific community as necessary to validate research findings” be made available at little or no cost to the PI or project. In accordance with this policy and guidance from the Office of Management and Budget, this plan does not include preliminary analyses (including raw data), drafts of scientific papers, plans for future research, peer reviews, or communications with colleagues. Data that must be withheld long enough to enable peer review and publication/dissemination or protection of intellectual property is subject to this plan only after those steps have taken place. Under this application, we will determine the effectiveness the proposed nano-vesicles (NETs) as photo-theranostic materials for fluorescence imaging and photothermal therapies. The release of data about students or any other human subjects is subject to policies and restrictions in protocols adopted by the relevant Institutional Research Board (IRB) and the Family Educational Rights and Privacy Act (FERPA) regulations.</t>
+          <t>Overview</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>3. Data and Metadata Format and Contents</t>
+          <t>This Data Management Plan has been prepared in accordance with guidelines from the NSF Division of Chemistry, “Advice to PIs on Data Management Plans,” and is consistent with the NSF Policy on Dissemination and Sharing of Research Results.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>We will make the proposed nano-vesicles (NETs) available to interested investigators who would like to use them in their scientific research. We will publish our results, and present them results in relevant conferences, workshops, seminars, and teaching forums. Additionally, we will provide our results to any national resources and or databases on nanoparticles that compile and maintain such information. As an example, we will contribute to the nanotechnology information library (NIL) (http://nanoparticlelibrary.net/index.asp), which is maintained by the National Institute for Occupational Safety and Health (NIOSH). Data that must be withheld long enough to enable peer review and publication/dissemination or protection of intellectual property will be subject after appropriate steps have taken place. Confidential material will be handled according to policies and protocols at UCR, Family Educational Rights and Privacy Act (FERPA), and any other applicable regulations and restrictions. All materials uploaded to the eScholarship site will be tagged uniformly with metadata about the source and nature of the data. Any electronic file format (e.g., text, spreadsheets, images) can be accepted. As a service to assure that materials are formatted correctly, a curator from the College reviews all submissions before they are accepted.</t>
+          <t>Data Sharing Across Teams</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>4. Accessibility and Data Protection</t>
+          <t>The C-GEM team will store, share, disseminate, and archive data following well-established, open, effective, secure, and timely processes. At the core of our Data Management strategy is GEM-NET, a set of web tools that support virtual teamwork via a Google Team Drive that provides unlimited storage for presentations, documents, and other data, including the underlying data storage for our custom data management apps. These custom apps include: - Strains, which tracks the identity and transfer of strains and plasmids; - Protocols, which documents our laboratory procedures; and - Molecules (in progress), which houses information on the structures, synthesis, characterization, and team usage of C-GEM monomers. Future work will incorporate a “search by structure” capability to help users find monomers quickly even when the archive scales to thousands of entries. We will also develop a searchable archive of GEM-NET Laboratory Notebooks that document research and can be associated with specific records in our Protocols, Strains, and Molecules databases. All new team members will receive a GEM-NET orientation to help them become rapidly proficient in each of these tools.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Materials will be searchable through a number of databases and search engines, including Google and Google Scholar. As noted in Section 2 (Scope), data will be made available only after appropriate steps have been taken to protect intellectual property. Confidential material will be handled according to policies and protocols for human subjects, FERPA, and any other applicable regulations and restrictions. Stored materials are downloadable but not editable, and they are backed up to assure no loss of data. All uploads are approved by a curator before they are published.</t>
+          <t>1. C-GEM Research Products</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>5. Derivative Products</t>
+          <t>(A) Materials. C-GEM scientists will produce new chemical compounds, new biological reagents, and new bacterial strains.
+(B) Experimental Data. Data will be collected from chemical synthesis procedures, biochemical, structural, and molecular biology experiments, and structural and functional characterization of C-GEM polymers. Such data include spectra, chromatograms, diffraction data, images, and results of properties analysis. Metadata will be generated describing the storage locations of chemical compounds, plasmids, and bacterial strains. We will also generate annotations of various sequence information (polymers, proteins, DNA).
+(C) Software. We will generate software including custom GEM-NET apps written in Python, algorithms for the Rosetta molecular modeling software suite, and simulation programs.
+(D) Other Products. We will generate experimental protocols and collect data on GEM-NET usage from component services.
+(E) Education and Outreach Materials. Our broader impacts and public engagement activities will generate educational materials (syllabi, lectures, demonstrations, hands-on activities) and online content (videos, blog posts, podcasts).
+(F) Evaluation Data. Our management and broader impact activities will generate assessments, narratives, and aggregated information about participants. Human subject protocols will be developed and submitted for IRB review/approval at each institution pending notice of award.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>All materials will contain acknowledgement of NSF support as per NSF policy: “ This material is based upon work supported by the National Science Foundation under Grant No. (NSF grant number). ” Additionally, materials will contain a disclaimer that “ any opinions, findings, and conclusions or recommendations expressed in this material are those of the author(s) and do not necessarily reflect the views of the National Science Foundation .” In keeping with standard ethical practices, it is expected that subsequent users of the data will acknowledge the source.</t>
+          <t>2. Data Format</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>6. Archiving and Access</t>
+          <t>Collected data will be formatted in several ways: (A) images as .tiff files; (B) experimental data as csv/Excel files or more specialized formats from the output of FACS, LC-MS, cryo-EM, etc.; and (C) laboratory protocols and notes, initially as pdfs or images scanned from lab notebooks, and then in a common GEM-NET Notebook format. Whenever possible, we will save data in machine-readable non-proprietary formats; in cases where that is not possible, we will provide images or extracted data to interested parties upon request.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>sample10</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>It is understood that the NSF Engineering Directorate requires data to be made available for a minimum of three years after conclusion of the award or public release, whichever is later. If the PI leaves his institution, the products will remain stored in relevant databases. PI is free to reproduce and repost these materials at new institution.</t>
+          <t>3. Access to Data and Data Sharing Practices and Policies</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>sample11</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>3.3.3 Data Management Plan</t>
+          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines. (B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs). (C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice. (D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website. (E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication. (F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>sample11</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>All participants in the proposed project with access to the numerical codes and computational data will conform closely to NASA policy on preserving and sharing of the research data and gathered in the course of the proposed project. The data acquired and preserved in the context of this proposal will be further governed by UCSB’s policies pertaining to intellectual property, record retention, and data management.</t>
+          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>sample11</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -2958,24 +2977,24 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Digital products from this project include: 1) a numerical code that can predict the ADR performance of a magnetic refrigerant based on DFT and DFPT simulation of magnon and phonon properties. The computer code will be published on the open-source website GitHub. PI Liao has published homemade code on GitHub before (https://github.com/nanoengineering/EPW-nano). 2) a numerical code that solves the coupled magnon-phonon Boltzmann transport equations. This software will be written in Python and published and regularly maintained/updated on the open-source website GitHub. 3) Data from first-principles simulations, including magnon and phonon transport properties of selected magnetic materials. Metadata that describes simulation conditions will also be generated, indexed, and archived together with the raw data. Raw simulation data will be carefully curated and archived. The team will archive all data in local computers and a centralized data storage system based on external hard drives, which is synchronized to cloud storage (UCSB provides unlimited Google Drive storage space to researchers). Graduate students participating in this project will be directly responsible for collecting, curating, and archiving the data. They will be trained by PI Liao before the start of the project on the proper protocol of handling data. The stored data will be periodically (at least monthly) inspected by PI Liao. In the event of the departure of key personnel, a written document detailing the content and the condition of the data that they are responsible for should be prepared and data transfer and training should be conducted before the departure.</t>
+          <t>The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan. (A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access. (B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>sample11</t>
+          <t>sample12</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>We will publish primary results expeditiously in peer-reviewed journals, supported by relevant data in the supplementary documents along with the published papers. Raw data supporting published papers will be made available to the public automatically by depositing the data to the open-access repository Figshare, and the web link will be provided in the published paper. The raw data will be properly annotated and detailed metadata that describes the content, format, organization of the raw data will also be provided to help interpret the raw data. If processed data is used in the publication, the processing procedure will be described in detail in the paper. We will provide full assistance in terms of raw data availability, data processing software and error analysis for other researchers to validate and reproduce our results. We will make peer-reviewed publications from this project all available to the public by depositing the accepted manuscripts to depositories like arXiv and PubMed Central.</t>
+          <t>5. Archival Storage Standards</t>
         </is>
       </c>
     </row>
@@ -2987,121 +3006,123 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>C-GEM: Plan for Data Management</t>
+          <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive. (A) Timing. Data will be archived within 1 month of validation or upon publication. (B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley. (C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Understanding the protein composition and dynamics of the nuclear envelope in plants</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>This Data Management Plan has been prepared in accordance with guidelines from the NSF Division of Chemistry, “Advice to PIs on Data Management Plans,” and is consistent with the NSF Policy on Dissemination and Sharing of Research Results.</t>
+          <t>DATA MANAGEMENT PLAN
+PI Gu</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Data Sharing Across Teams</t>
+          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>The C-GEM team will store, share, disseminate, and archive data following well-established, open, effective, secure, and timely processes. At the core of our Data Management strategy is GEM-NET, a set of web tools that support virtual teamwork via a Google Team Drive that provides unlimited storage for presentations, documents, and other data, including the underlying data storage for our custom data management apps. These custom apps include: - Strains, which tracks the identity and transfer of strains and plasmids; - Protocols, which documents our laboratory procedures; and - Molecules (in progress), which houses information on the structures, synthesis, characterization, and team usage of C-GEM monomers. Future work will incorporate a “search by structure” capability to help users find monomers quickly even when the archive scales to thousands of entries. We will also develop a searchable archive of GEM-NET Laboratory Notebooks that document research and can be associated with specific records in our Protocols, Strains, and Molecules databases. All new team members will receive a GEM-NET orientation to help them become rapidly proficient in each of these tools.</t>
+          <t>Proteomic Data</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>1. C-GEM Research Products</t>
+          <t>Description
+This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>(A) Materials. C-GEM scientists will produce new chemical compounds, new biological reagents, and new bacterial strains.</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -3111,65 +3132,67 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>(B) Experimental Data. Data will be collected from chemical synthesis procedures, biochemical, structural, and molecular biology experiments, and structural and functional characterization of C-GEM polymers. Such data include spectra, chromatograms, diffraction data, images, and results of properties analysis. Metadata will be generated describing the storage locations of chemical compounds, plasmids, and bacterial strains. We will also generate annotations of various sequence information (polymers, proteins, DNA).</t>
+          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.
+Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>(C) Software. We will generate software including custom GEM-NET apps written in Python, algorithms for the Rosetta molecular modeling software suite, and simulation programs.</t>
+          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>(D) Other Products. We will generate experimental protocols and collect data on GEM-NET usage from component services.</t>
+          <t>Description
+This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>(E) Education and Outreach Materials. Our broader impacts and public engagement activities will generate educational materials (syllabi, lectures, demonstrations, hands-on activities) and online content (videos, blog posts, podcasts).</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -3179,14 +3202,14 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>(F) Evaluation Data. Our management and broader impact activities will generate assessments, narratives, and aggregated information about participants. Human subject protocols will be developed and submitted for IRB review/approval at each institution pending notice of award.</t>
+          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -3196,31 +3219,32 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2. Data Format</t>
+          <t>Publications</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Collected data will be formatted in several ways: (A) images as .tiff files; (B) experimental data as csv/Excel files or more specialized formats from the output of FACS, LC-MS, cryo-EM, etc.; and (C) laboratory protocols and notes, initially as pdfs or images scanned from lab notebooks, and then in a common GEM-NET Notebook format. Whenever possible, we will save data in machine-readable non-proprietary formats; in cases where that is not possible, we will provide images or extracted data to interested parties upon request.</t>
+          <t>Description
+Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -3230,14 +3254,14 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>3. Access to Data and Data Sharing Practices and Policies</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -3247,14 +3271,14 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines. (B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs). (C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice. (D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website. (E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication. (F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
+          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -3264,31 +3288,32 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives</t>
+          <t>Teaching Curricula</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan. (A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access. (B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
+          <t>Description
+Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -3298,14 +3323,14 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>5. Archival Storage Standards</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>sample12</t>
+          <t>sample13</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -3314,431 +3339,6 @@
         </is>
       </c>
       <c r="C169" t="inlineStr">
-        <is>
-          <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive. (A) Timing. Data will be archived within 1 month of validation or upon publication. (B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley. (C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>Understanding the protein composition and dynamics of the nuclear envelope in plants</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>DATA MANAGEMENT PLAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>PI Gu</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>Proteomic Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>Archiving and Dissemination</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>Archiving and Dissemination</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>Publications</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>Archiving and Dissemination</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>Teaching Curricula</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>Archiving and Dissemination</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>sample13</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="C194" t="inlineStr">
         <is>
           <t>Lectures, student presentations, data collection, training resources will be maintained online through the UC Berkeley bCourses course management system and backed up online through the unlimited cloud-based storage space offered by Google.</t>
         </is>
@@ -4103,7 +3703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4154,19 +3754,8 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Digital products from this project include: 1) a numerical code that can predict the ADR performance of a magnetic refrigerant based on DFT and DFPT simulation of magnon and phonon properties. The computer code will be published on the open-source website GitHub. PI Liao has published homemade code on GitHub before (https://github.com/nanoengineering/EPW-nano). 2) a numerical code that solves the coupled magnon-phonon Boltzmann transport equations. This software will be written in Python and published and regularly maintained/updated on the open-source website GitHub. 3) Data from first-principles simulations, including magnon and phonon transport properties of selected magnetic materials. Metadata that describes simulation conditions will also be generated, indexed, and archived together with the raw data. Raw simulation data will be carefully curated and archived. The team will archive all data in local computers and a centralized data storage system based on external hard drives, which is synchronized to cloud storage (UCSB provides unlimited Google Drive storage space to researchers). Graduate students participating in this project will be directly responsible for collecting, curating, and archiving the data. They will be trained by PI Liao before the start of the project on the proper protocol of handling data. The stored data will be periodically (at least monthly) inspected by PI Liao. In the event of the departure of key personnel, a written document detailing the content and the condition of the data that they are responsible for should be prepared and data transfer and training should be conducted before the departure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>We will publish primary results expeditiously in peer-reviewed journals, supported by relevant data in the supplementary documents along with the published papers. Raw data supporting published papers will be made available to the public automatically by depositing the data to the open-access repository Figshare, and the web link will be provided in the published paper. The raw data will be properly annotated and detailed metadata that describes the content, format, organization of the raw data will also be provided to help interpret the raw data. If processed data is used in the publication, the processing procedure will be described in detail in the paper. We will provide full assistance in terms of raw data availability, data processing software and error analysis for other researchers to validate and reproduce our results. We will make peer-reviewed publications from this project all available to the public by depositing the accepted manuscripts to depositories like arXiv and PubMed Central.</t>
+          <t>Digital products from this project include: 1) a numerical code that can predict the ADR performance of a magnetic refrigerant based on DFT and DFPT simulation of magnon and phonon properties. The computer code will be published on the open-source website GitHub. PI Liao has published homemade code on GitHub before (https://github.com/nanoengineering/EPW-nano). 2) a numerical code that solves the coupled magnon-phonon Boltzmann transport equations. This software will be written in Python and published and regularly maintained/updated on the open-source website GitHub. 3) Data from first-principles simulations, including magnon and phonon transport properties of selected magnetic materials. Metadata that describes simulation conditions will also be generated, indexed, and archived together with the raw data. Raw simulation data will be carefully curated and archived. The team will archive all data in local computers and a centralized data storage system based on external hard drives, which is synchronized to cloud storage (UCSB provides unlimited Google Drive storage space to researchers). Graduate students participating in this project will be directly responsible for collecting, curating, and archiving the data. They will be trained by PI Liao before the start of the project on the proper protocol of handling data. The stored data will be periodically (at least monthly) inspected by PI Liao. In the event of the departure of key personnel, a written document detailing the content and the condition of the data that they are responsible for should be prepared and data transfer and training should be conducted before the departure.
+We will publish primary results expeditiously in peer-reviewed journals, supported by relevant data in the supplementary documents along with the published papers. Raw data supporting published papers will be made available to the public automatically by depositing the data to the open-access repository Figshare, and the web link will be provided in the published paper. The raw data will be properly annotated and detailed metadata that describes the content, format, organization of the raw data will also be provided to help interpret the raw data. If processed data is used in the publication, the processing procedure will be described in detail in the paper. We will provide full assistance in terms of raw data availability, data processing software and error analysis for other researchers to validate and reproduce our results. We will make peer-reviewed publications from this project all available to the public by depositing the accepted manuscripts to depositories like arXiv and PubMed Central.</t>
         </is>
       </c>
     </row>
@@ -4181,7 +3770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4280,19 +3869,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>(A) Materials. C-GEM scientists will produce new chemical compounds, new biological reagents, and new bacterial strains.</t>
+          <t>(A) Materials. C-GEM scientists will produce new chemical compounds, new biological reagents, and new bacterial strains.
+(B) Experimental Data. Data will be collected from chemical synthesis procedures, biochemical, structural, and molecular biology experiments, and structural and functional characterization of C-GEM polymers. Such data include spectra, chromatograms, diffraction data, images, and results of properties analysis. Metadata will be generated describing the storage locations of chemical compounds, plasmids, and bacterial strains. We will also generate annotations of various sequence information (polymers, proteins, DNA).
+(C) Software. We will generate software including custom GEM-NET apps written in Python, algorithms for the Rosetta molecular modeling software suite, and simulation programs.
+(D) Other Products. We will generate experimental protocols and collect data on GEM-NET usage from component services.
+(E) Education and Outreach Materials. Our broader impacts and public engagement activities will generate educational materials (syllabi, lectures, demonstrations, hands-on activities) and online content (videos, blog posts, podcasts).
+(F) Evaluation Data. Our management and broader impact activities will generate assessments, narratives, and aggregated information about participants. Human subject protocols will be developed and submitted for IRB review/approval at each institution pending notice of award.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>(B) Experimental Data. Data will be collected from chemical synthesis procedures, biochemical, structural, and molecular biology experiments, and structural and functional characterization of C-GEM polymers. Such data include spectra, chromatograms, diffraction data, images, and results of properties analysis. Metadata will be generated describing the storage locations of chemical compounds, plasmids, and bacterial strains. We will also generate annotations of various sequence information (polymers, proteins, DNA).</t>
+          <t>2. Data Format</t>
         </is>
       </c>
     </row>
@@ -4304,19 +3898,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>(C) Software. We will generate software including custom GEM-NET apps written in Python, algorithms for the Rosetta molecular modeling software suite, and simulation programs.</t>
+          <t>Collected data will be formatted in several ways: (A) images as .tiff files; (B) experimental data as csv/Excel files or more specialized formats from the output of FACS, LC-MS, cryo-EM, etc.; and (C) laboratory protocols and notes, initially as pdfs or images scanned from lab notebooks, and then in a common GEM-NET Notebook format. Whenever possible, we will save data in machine-readable non-proprietary formats; in cases where that is not possible, we will provide images or extracted data to interested parties upon request.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>(D) Other Products. We will generate experimental protocols and collect data on GEM-NET usage from component services.</t>
+          <t>3. Access to Data and Data Sharing Practices and Policies</t>
         </is>
       </c>
     </row>
@@ -4328,113 +3922,53 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>(E) Education and Outreach Materials. Our broader impacts and public engagement activities will generate educational materials (syllabi, lectures, demonstrations, hands-on activities) and online content (videos, blog posts, podcasts).</t>
+          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines. (B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs). (C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice. (D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website. (E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication. (F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>(F) Evaluation Data. Our management and broader impact activities will generate assessments, narratives, and aggregated information about participants. Human subject protocols will be developed and submitted for IRB review/approval at each institution pending notice of award.</t>
+          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2. Data Format</t>
+          <t>The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan. (A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access. (B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Collected data will be formatted in several ways: (A) images as .tiff files; (B) experimental data as csv/Excel files or more specialized formats from the output of FACS, LC-MS, cryo-EM, etc.; and (C) laboratory protocols and notes, initially as pdfs or images scanned from lab notebooks, and then in a common GEM-NET Notebook format. Whenever possible, we will save data in machine-readable non-proprietary formats; in cases where that is not possible, we will provide images or extracted data to interested parties upon request.</t>
+          <t>5. Archival Storage Standards</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
-        <is>
-          <t>3. Access to Data and Data Sharing Practices and Policies</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>(A) Intellectual Property, copyrights, and data will be administered in accordance with the policies of NSF and the participating institution(s) and codified in the C-GEM Collaboration Agreement. We expect all researchers to respect their responsibilities to the chemical and broader scientific communities and provide their results, data, and collections to other researchers upon request and in accordance with all university guidelines. (B) Materials will be disseminated in accordance with participating institutional and NSF policies. Depending on the terms of those policies, materials may be transferred to others under Material Transfer Agreements (MTAs). (C) Research Data will be made available after the findings have been accepted for publication. Research products will be preserved for open access wherever possible. Structural data will be deposited in the appropriate database upon publication, following standard practice. (D) Software. Source code for custom GEM-NET apps will be distributed through GitHub. Rosetta algorithms will be made available on the Rosetta Commons. The SCA4RNA algorithm will be made available on the C-GEM website. (E) Publications. C-GEM investigators will promptly prepare and submit manuscripts resulting from NSF support, assign authorship to accurately reflect contributions, and acknowledge funding support in accordance with agency policies. Our Code of Conduct encourages submission of pre-prints prior to publication. (F) EteRNA. Citizen scientists who engage in C-GEM×EteRNA design challenges will access project data in a convenient, searchable format through the EteRNA lab visualizer after registration (free of charge) with the EteRNA project (http://eternagame.org). Under the EteRNA User Agreement, players relinquish any IP claims and consent to sharing their designs with collaborators. The EteRNA project (and individual players, when appropriate) will receive authorship and/or acknowledgement on C-GEM publications following established norms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>4. Policies for Re-use, Re-distribution, and Production of Derivatives</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>The Director has overall responsibility for both data management and dissemination. C-GEM Investigators will share with other researchers, at no more than incremental cost and within reasonable time, the primary data, samples, physical collections, software, curriculum materials, and other supporting materials created or gathered in the course of NSF-funded work. Each collaborator will sign a Collaboration Agreement pledging to abide by the terms of this Data Management Plan. (A) Sensitive data will be made available to the Director, Center staff, and select members of the External Advisory Board with relevant expertise. Privacy, confidentiality, and security of personal data collected for evaluation will be ensured via the following standard practices: collecting data anonymously (through Google Forms); refraining from collection of demographic data that could render individuals identifiable; and storing sensitive data on a separate password- protected GEM-NET Team Drive with limited access. (B) Materials for general access will be shared on the C-GEM website (educational materials, blog posts, resources) under a CC BY-NC-SA 3.0 license that allows users to share and adapt material for noncommercial use, requires attribution, and requires any new material created to be distributed under the same terms. Podcasts are disseminated through Yale University on Apple Podcasts and SoundCloud (CC BY-NC-SA 3.0 license).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>5. Archival Storage Standards</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
         <is>
           <t>Preliminary data will be stored on office computers and local data systems accessible from workstations associated with each C-GEM Investigator. Data in non-electronic form will be converted to digital form for preservation. Final responsibility for data archiving and preservation lies with each Investigator. At the conclusion of the grant, data can be maintained indefinitely on local backups and also, for as long as C-GEM exists as an educational entity, on the Team Drive. (A) Timing. Data will be archived within 1 month of validation or upon publication. (B) Method of Archiving. Data will be uploaded to a “Data” Team Drive, the contents of which will be backed up weekly to a local server at UC-Berkeley. (C) Preservation of Access. Access to Team Drive and GEM-NET apps is provisioned to individual google accounts. We will use Google Groups for access control and will create an “alumni” group for former C-GEM members with read-only permissions. If necessary, we can create GEM-NET.net Google accounts for departing members.</t>
         </is>
@@ -4451,7 +3985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4490,67 +4024,70 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DATA MANAGEMENT PLAN</t>
+          <t>DATA MANAGEMENT PLAN
+PI Gu</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PI Gu</t>
+          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
+          <t>Proteomic Data</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Proteomic Data</t>
+          <t>Description
+This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
+          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.
+Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
         </is>
       </c>
     </row>
@@ -4562,55 +4099,56 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Archiving and Dissemination</t>
+          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.</t>
+          <t>Description
+This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
+          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Publications</t>
         </is>
       </c>
     </row>
@@ -4622,7 +4160,8 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
+          <t>Description
+Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4185,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
+          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4197,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Publications</t>
+          <t>Teaching Curricula</t>
         </is>
       </c>
     </row>
@@ -4670,101 +4209,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Description
+Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
+          <t>Archiving and Dissemination</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
-        <is>
-          <t>Archiving and Dissemination</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Teaching Curricula</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Archiving and Dissemination</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
         <is>
           <t>Lectures, student presentations, data collection, training resources will be maintained online through the UC Berkeley bCourses course management system and backed up online through the unlimited cloud-based storage space offered by Google.</t>
         </is>
@@ -5147,7 +4615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5282,19 +4750,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>All data pertaining to any published work will be made available to any person on request. Numerical published data as well as the original raw data files will be freely accessible either as supplementary data files included with published papers, or as files posted on the web sites of the laboratories in the Center. Additional data or programs required by third parties will be provided on request. Data that may support intellectual property claims will be published only after we seek advice from the Northwestern Innovation and New Ventures Office (INVO). Such advice will be sought in a timely manner. Otherwise, there are no restrictions on who will be allowed to use the data generated after publishing is complete, provided that the requester acknowledges the original work. A requester can use data output of our work, provided guidelines by the publisher for use of published data are followed.</t>
+          <t>All data pertaining to any published work will be made available to any person on request. Numerical published data as well as the original raw data files will be freely accessible either as supplementary data files included with published papers, or as files posted on the web sites of the laboratories in the Center. Additional data or programs required by third parties will be provided on request. Data that may support intellectual property claims will be published only after we seek advice from the Northwestern Innovation and New Ventures Office (INVO). Such advice will be sought in a timely manner. Otherwise, there are no restrictions on who will be allowed to use the data generated after publishing is complete, provided that the requester acknowledges the original work. A requester can use data output of our work, provided guidelines by the publisher for use of published data are followed.
+Electronic files are stored on secure servers hosted by the individual research groups and safeguarded by automated backup systems and/or backups to off-site servers maintained by their institution. We project that all of these systems will be in place for at least 10 years. All non-electronic data including detailed experimental procedures and observations are recorded in laboratory notebooks that do not leave the senior investigator's lab. Data should be accessible to the rest of the laboratory, but access is typically revoked when junior investigators leave the lab.
+Data will also be deposited into Northwestern Libraries’ institutional repository, Arch, upon publication. https://arch.library.northwestern.edu/ Arch assigns DOIs, making it easy to find the data. Necessary metadata and other resources to make the data accessible to future users will be submitted. Arch will preserve the data for future use. External investigators may choose to instead archive their data with similar repositories provided by the partner institution (such as Academic Commons at Columbia University, D-Scholarship@Pitt at the University of Pittsburgh, and Harvard University Archives).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Electronic files are stored on secure servers hosted by the individual research groups and safeguarded by automated backup systems and/or backups to off-site servers maintained by their institution. We project that all of these systems will be in place for at least 10 years. All non-electronic data including detailed experimental procedures and observations are recorded in laboratory notebooks that do not leave the senior investigator's lab. Data should be accessible to the rest of the laboratory, but access is typically revoked when junior investigators leave the lab.</t>
+          <t>Rationale. A discussion of the rationale or justification for the proposed data management plan including, for example, the potential impact of the data within the immediate field and in other fields, and any broader societal impact.</t>
         </is>
       </c>
     </row>
@@ -5306,67 +4776,68 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data will also be deposited into Northwestern Libraries’ institutional repository, Arch, upon publication. https://arch.library.northwestern.edu/ Arch assigns DOIs, making it easy to find the data. Necessary metadata and other resources to make the data accessible to future users will be submitted. Arch will preserve the data for future use. External investigators may choose to instead archive their data with similar repositories provided by the partner institution (such as Academic Commons at Columbia University, D-Scholarship@Pitt at the University of Pittsburgh, and Harvard University Archives).</t>
+          <t>The Department of Energy stipulates in their "Statement on Digital Data Management" that "To the greatest extent and with the fewest constraints possible, and consistent with the requirements and other principles of this Statement, data sharing should make digital research data available to and useful for the scientific community, industry, and the public." The Center will make every effort to comply with these guidelines. Data that is not deemed to be useful for a publication may still be archived at the discretion of the senior investigator overseeing the work, taking into the costs and benefits of doing so. The data acquired and preserved in the context of this proposal will be further governed by policies of the Northwestern University and its partner institutions pertaining to intellectual property, record retention, and data management.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Rationale. A discussion of the rationale or justification for the proposed data management plan including, for example, the potential impact of the data within the immediate field and in other fields, and any broader societal impact.</t>
+          <t>2. Data used in publications</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>The Department of Energy stipulates in their "Statement on Digital Data Management" that "To the greatest extent and with the fewest constraints possible, and consistent with the requirements and other principles of this Statement, data sharing should make digital research data available to and useful for the scientific community, industry, and the public." The Center will make every effort to comply with these guidelines. Data that is not deemed to be useful for a publication may still be archived at the discretion of the senior investigator overseeing the work, taking into the costs and benefits of doing so. The data acquired and preserved in the context of this proposal will be further governed by policies of the Northwestern University and its partner institutions pertaining to intellectual property, record retention, and data management.</t>
+          <t>Data management plans should provide a plan for making all research data displayed in publications resulting from the proposed research open, machine-readable, and digitally accessible to the public at the time of publication. This includes data that are displayed in charts, figures, images, etc. In addition, the underlying digital research data used to generate the displayed data should be made as accessible as possible to the public in accordance with the Principles published in the DOE Policy for Digital Research Data Management. The published article should indicate how these data can be accessed.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2. Data used in publications</t>
+          <t>Research conducted within the Center will be published in appropriate scientific journals. The publisher may restrict the redistribution of that data. When not prohibitively expensive, open access will be selected. This will be supplemented by publishing the data in a preprint repository such as the arXiv subsequent to peer-reviewed publication if possible. All publishers we previously worked with allow arXiv publication or open access, so we do not anticipate a problem. Crystallographic data will be deposited into the ICSD or the CCDC databases for broad access. Data will also be disseminated through seminars at conferences and at other academic institutions. Raw data files can be provided to others upon request, but will be limited to their personal use only and cannot be redistributed without written consent from the PI.
+Access to data and results prior to publication or file for intellectual property is provided to all personnel involved in the project, after publication or filing for provisional patents, the data will be in the public domain and any further data will be provided to the community upon request or through appropriate websites (i.e. lab web sites). All of the fabrication methods, characterization results, and data acquired through the proposed research towards the development of the bioactive platforms will be shared with others through publication in conferences and journals.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Data management plans should provide a plan for making all research data displayed in publications resulting from the proposed research open, machine-readable, and digitally accessible to the public at the time of publication. This includes data that are displayed in charts, figures, images, etc. In addition, the underlying digital research data used to generate the displayed data should be made as accessible as possible to the public in accordance with the Principles published in the DOE Policy for Digital Research Data Management. The published article should indicate how these data can be accessed.</t>
+          <t>3. Data management resources</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Research conducted within the Center will be published in appropriate scientific journals. The publisher may restrict the redistribution of that data. When not prohibitively expensive, open access will be selected. This will be supplemented by publishing the data in a preprint repository such as the arXiv subsequent to peer-reviewed publication if possible. All publishers we previously worked with allow arXiv publication or open access, so we do not anticipate a problem. Crystallographic data will be deposited into the ICSD or the CCDC databases for broad access. Data will also be disseminated through seminars at conferences and at other academic institutions. Raw data files can be provided to others upon request, but will be limited to their personal use only and cannot be redistributed without written consent from the PI.</t>
+          <t>Data management plans should consult and reference available information about data management resources to be used in the course of the proposed research. In particular, DMPs tht explicitly or implicitly commit data management resources at a facility beyond what is conventionally made available to approved users should be accompanied by written approval from that facility. In determining the resources available for data management at DOE Scientific User Facilities, researchers should consult the published description of data management resources and practices at that facility and reference it in the DMP. Information about other Office of Science facilities can be found in the additional guidance from the sponsporing program.</t>
         </is>
       </c>
     </row>
@@ -5378,7 +4849,9 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Access to data and results prior to publication or file for intellectual property is provided to all personnel involved in the project, after publication or filing for provisional patents, the data will be in the public domain and any further data will be provided to the community upon request or through appropriate websites (i.e. lab web sites). All of the fabrication methods, characterization results, and data acquired through the proposed research towards the development of the bioactive platforms will be shared with others through publication in conferences and journals.</t>
+          <t>DMPs should consult and reference available information about data management resources to be used in the course of the proposed research. In particular, DMPs that explicitly or implicitly commit data management resources at a facility beyond what is conventionally made available to approved users should be accompanied by written approval from that facility. In determining the resources available for data management at Office of Science User Facilities, researchers should consult the published description of data management resources and practices at that facility and reference it in the DMP. Information about other Office of Science facilities can be found in the additional guidance from the sponsoring program.
+Data Repositories. Senior investigators typically archive relevant data using their own group servers. Whenever possible, investigators will be encouraged to also copy data to a centralized data server for CBES investigators. Additionally, researchers can archive data on repositories at their home institutions. For example, researchers at Northwestern are encouraged to deposit data into Northwestern Libraries’ institutional repository, Arch, upon publication (https://arch.library.northwestern.edu/). Arch assigns DOIs, making it easy to find the data. Necessary metadata and other resources to make the data accessible to future users will be submitted. Arch will preserve the data for future use.
+Data Volume. Generally, the volume of data generated by CBES researchers should not prohibit their deposition in available repositories. However, in cases where large volumes of data are generated (e.g., temperature/time dependent microscopy or X-ray studies), the data may need to be averaged, condensed, or minimally processed prior to deposition.</t>
         </is>
       </c>
     </row>
@@ -5390,7 +4863,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3. Data management resources</t>
+          <t>4. Confidentiality, security and rights</t>
         </is>
       </c>
     </row>
@@ -5402,7 +4875,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Data management plans should consult and reference available information about data management resources to be used in the course of the proposed research. In particular, DMPs tht explicitly or implicitly commit data management resources at a facility beyond what is conventionally made available to approved users should be accompanied by written approval from that facility. In determining the resources available for data management at DOE Scientific User Facilities, researchers should consult the published description of data management resources and practices at that facility and reference it in the DMP. Information about other Office of Science facilities can be found in the additional guidance from the sponsporing program.</t>
+          <t>Data management plans must protect confidentiality, personal privacy, Personally Identifiable Information and U.S. national, homeland, and economic security; recognize proprietary interests, business confidential information, and intellectual property rights; avoid significant negative impact on innovation and U.S. competitiveness; and otherwise be consistent with all applicable laws, regulations, agreement terms and conditions, and DOE orders and policies. There is no requirement to share proprietary data.</t>
         </is>
       </c>
     </row>
@@ -5413,66 +4886,6 @@
         </is>
       </c>
       <c r="B22" t="inlineStr">
-        <is>
-          <t>DMPs should consult and reference available information about data management resources to be used in the course of the proposed research. In particular, DMPs that explicitly or implicitly commit data management resources at a facility beyond what is conventionally made available to approved users should be accompanied by written approval from that facility. In determining the resources available for data management at Office of Science User Facilities, researchers should consult the published description of data management resources and practices at that facility and reference it in the DMP. Information about other Office of Science facilities can be found in the additional guidance from the sponsoring program.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Data Repositories. Senior investigators typically archive relevant data using their own group servers. Whenever possible, investigators will be encouraged to also copy data to a centralized data server for CBES investigators. Additionally, researchers can archive data on repositories at their home institutions. For example, researchers at Northwestern are encouraged to deposit data into Northwestern Libraries’ institutional repository, Arch, upon publication (https://arch.library.northwestern.edu/). Arch assigns DOIs, making it easy to find the data. Necessary metadata and other resources to make the data accessible to future users will be submitted. Arch will preserve the data for future use.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Data Volume. Generally, the volume of data generated by CBES researchers should not prohibit their deposition in available repositories. However, in cases where large volumes of data are generated (e.g., temperature/time dependent microscopy or X-ray studies), the data may need to be averaged, condensed, or minimally processed prior to deposition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>4. Confidentiality, security and rights</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Data management plans must protect confidentiality, personal privacy, Personally Identifiable Information and U.S. national, homeland, and economic security; recognize proprietary interests, business confidential information, and intellectual property rights; avoid significant negative impact on innovation and U.S. competitiveness; and otherwise be consistent with all applicable laws, regulations, agreement terms and conditions, and DOE orders and policies. There is no requirement to share proprietary data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
         <is>
           <t>Data that may support intellectual property claims will be published only after we seek advice from the Northwestern Innovation and New Ventures Office (INVO). Such advice will be sought in a timely manner. The proposed research does not include the collection of any confidential personal information. The Director, the Executive Director for Research, and the Executive Committee will regularly review polices for data storage to ensure accessibility and security of CBES research data.</t>
         </is>
@@ -5741,7 +5154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5804,55 +5217,59 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Section 2.1 characterizes the aquifer formation that each groundwater well in the West taps and compares well construction patterns before and after the establishment of regulatory controls.</t>
+          <t>Section 2.1 characterizes the aquifer formation that each groundwater well in the West taps and compares well construction patterns before and after the establishment of regulatory controls.
+Section 2.2 estimates groundwater components of the water budget (withdrawals and consumption) yearly (2016-2021) at the field scale.
+Section 2.3 integrates research and education through the Scientist Spotlight and Hydrologic Sciences Workshops.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Section 2.2 estimates groundwater components of the water budget (withdrawals and consumption) yearly (2016-2021) at the field scale.</t>
+          <t>TYPES OF DATA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Section 2.3 integrates research and education through the Scientist Spotlight and Hydrologic Sciences Workshops.</t>
+          <t>The PI and PhD student will be responsible for all data-related activities including: collection, documentation and metadata description, quality control, storage and backup, archiving, and sharing.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TYPES OF DATA</t>
+          <t>The project will result in new sets of data, code, and tools. These outputs include: (a) source code to quality control, collate, and merge datasets, (b) open source models and budgets in R and/or python, and (c) sharable instructional materials (Scientist Spotlight activities and workshop materials).
+Input data: Available data will be systematically reviewed and downloaded. These data are likely available in the form of Microsoft Access files or Microsoft Excel spreadsheets; shapefiles or raster files; or text files or comma-delimited files. A multi-tier storage and quality assurance methodology will be adopted and will likely evolve as new datasets provide for challenging formats and organization.
+Produced Data: Datasets will be produced in Sections 2.1-2.3 of the proposal. These datasets will be formatted and shared in an open format (e.g., CSV) or in illustrator files (i.e., cross sections).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>The PI and PhD student will be responsible for all data-related activities including: collection, documentation and metadata description, quality control, storage and backup, archiving, and sharing.</t>
+          <t>DATA AND METADATA STANDARDS</t>
         </is>
       </c>
     </row>
@@ -5864,19 +5281,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>The project will result in new sets of data, code, and tools. These outputs include: (a) source code to quality control, collate, and merge datasets, (b) open source models and budgets in R and/or python, and (c) sharable instructional materials (Scientist Spotlight activities and workshop materials).</t>
+          <t>The data will be shared along with a README.txt, which will describe all files, their relationships, naming conventions, etc. Data elements and attributes will be described following ISO 19115 specifications and metadata schema and standards in Hydrology (e.g., following any establish standards of the Water Information Coordination Program’s Open Water Data Initiative (Larsen et al., 2016)) to allow for better interpretability and interoperability. Code and scripts produced in R and/or python will be documented for reproducibility purposes. The metadata for the codes will include: (1) description of the functions required to operate the analyses; (2) description of input parameters and outputs; and (3) test case, files and plots documenting the expected response of the model (Section 2.1) to a standard set of input parameters. Documentation will focus on the description of the functions, input parameters, outputs, the format of input data, instructions to run the model, and instructions to export the results. The outputs will be stored in CSV format with a metadata document describing the data structure of the output data.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Input data: Available data will be systematically reviewed and downloaded. These data are likely available in the form of Microsoft Access files or Microsoft Excel spreadsheets; shapefiles or raster files; or text files or comma-delimited files. A multi-tier storage and quality assurance methodology will be adopted and will likely evolve as new datasets provide for challenging formats and organization.</t>
+          <t>POLICIES FOR ACCESS AND SHARING</t>
         </is>
       </c>
     </row>
@@ -5888,55 +5305,58 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Produced Data: Datasets will be produced in Sections 2.1-2.3 of the proposal. These datasets will be formatted and shared in an open format (e.g., CSV) or in illustrator files (i.e., cross sections).</t>
+          <t>Raw data: Detailed information about how the data were obtained, including detailed contact information or websites for direct download and citations to all datasets will be provided to allow for accessibility and correct attribution to original collectors. All methodological procedures for data quality control and aggregation will be described in the data documentation. This information will be provided in the form of supplementary documentation for publications, in the README.txt file, and at the repository (record-level). All sharable raw data and the processed data will be archived in Dryad, https://datadryad.org, the agnostic open access repository backed by UCSB and the California Digital Library (CDL), which implements the latest best practices in data curation, publication, citation, and archival. Dryad assigns Digital Object Identifiers (DOIs) to deposited datasets and makes data discoverable through such services as the Thomson-Reuters Data Citation Index, Scopus, and Google Dataset Search. All data in Dryad is publicly accessible and released under a CC0 license. Data will be linked to publications and vice versa through DOIs.
+Scripts and code for analyses: All scripts and code will be archived in supplementary information appendices in publications as well as uploaded to Zenodo through the Dryad repository submission process along with the sharable raw and processed data in order to allow citations and a better connection to the research data curation and publication processes.
+Scientist spotlight: All scientist spotlight biographies, assignments, and open-access readings will be posted to an online Dashboard associated with the PI’s website, which is updated bi-monthly.
+Workshop frameworks: Workshop material will be shared with UCSB’s Diversity Committee through Google Drive; if workshop materials are fully supported by the Diversity Committee, these materials will also be shared through eSholarship for broader dissemination.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DATA AND METADATA STANDARDS</t>
+          <t>The PI is committed to publishing in open access journals. The UC is currently leading initiatives to assist faculty in paying for open access journals.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The data will be shared along with a README.txt, which will describe all files, their relationships, naming conventions, etc. Data elements and attributes will be described following ISO 19115 specifications and metadata schema and standards in Hydrology (e.g., following any establish standards of the Water Information Coordination Program’s Open Water Data Initiative (Larsen et al., 2016)) to allow for better interpretability and interoperability. Code and scripts produced in R and/or python will be documented for reproducibility purposes. The metadata for the codes will include: (1) description of the functions required to operate the analyses; (2) description of input parameters and outputs; and (3) test case, files and plots documenting the expected response of the model (Section 2.1) to a standard set of input parameters. Documentation will focus on the description of the functions, input parameters, outputs, the format of input data, instructions to run the model, and instructions to export the results. The outputs will be stored in CSV format with a metadata document describing the data structure of the output data.</t>
+          <t>POLICIES AND PROVISIONS FOR RE-USE, RE-DISTRIBUTION</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>POLICIES FOR ACCESS AND SHARING</t>
+          <t>All data deposited at Dryad will be publicly available under a CC0 license, meaning that others may freely build upon, enhance and reuse the works for any purposes without restriction under copyright or database law. CC0 does not exempt those who reuse the data from following community norms for scholarly communication, i.e., reusing the data in a way that is mindful of its limitations and citing the original data authors.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Raw data: Detailed information about how the data were obtained, including detailed contact information or websites for direct download and citations to all datasets will be provided to allow for accessibility and correct attribution to original collectors. All methodological procedures for data quality control and aggregation will be described in the data documentation. This information will be provided in the form of supplementary documentation for publications, in the README.txt file, and at the repository (record-level). All sharable raw data and the processed data will be archived in Dryad, https://datadryad.org, the agnostic open access repository backed by UCSB and the California Digital Library (CDL), which implements the latest best practices in data curation, publication, citation, and archival. Dryad assigns Digital Object Identifiers (DOIs) to deposited datasets and makes data discoverable through such services as the Thomson-Reuters Data Citation Index, Scopus, and Google Dataset Search. All data in Dryad is publicly accessible and released under a CC0 license. Data will be linked to publications and vice versa through DOIs.</t>
+          <t>PLANS FOR ARCHIVING AND PRESERVATION OF ACCESS</t>
         </is>
       </c>
     </row>
@@ -5948,103 +5368,8 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Scripts and code for analyses: All scripts and code will be archived in supplementary information appendices in publications as well as uploaded to Zenodo through the Dryad repository submission process along with the sharable raw and processed data in order to allow citations and a better connection to the research data curation and publication processes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Scientist spotlight: All scientist spotlight biographies, assignments, and open-access readings will be posted to an online Dashboard associated with the PI’s website, which is updated bi-monthly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Workshop frameworks: Workshop material will be shared with UCSB’s Diversity Committee through Google Drive; if workshop materials are fully supported by the Diversity Committee, these materials will also be shared through eSholarship for broader dissemination.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>The PI is committed to publishing in open access journals. The UC is currently leading initiatives to assist faculty in paying for open access journals.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>POLICIES AND PROVISIONS FOR RE-USE, RE-DISTRIBUTION</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>All data deposited at Dryad will be publicly available under a CC0 license, meaning that others may freely build upon, enhance and reuse the works for any purposes without restriction under copyright or database law. CC0 does not exempt those who reuse the data from following community norms for scholarly communication, i.e., reusing the data in a way that is mindful of its limitations and citing the original data authors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>PLANS FOR ARCHIVING AND PRESERVATION OF ACCESS</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>UCSB Box will be used as the primary means to store and back up all collected input, generated output data sets and code, and educational materials over the course of the project and prior to data sharing. Box provides encryption of data at rest and in-transit, detailed logging of file actions, two-factor authentication, and access review of collaborators. Data will be accessed using Box Drive, which requires full disk encryption, firewall, and an antivirus software in order to install on a local computer. At the end of the project, all shareable data accompanied by the appropriate documentation, metadata, and code will be deposited into Dryad for long-term storage, preservation and accessibility. Deposits submitted to Dryad are curated prior to public release to conform with quality standards and enable future reuse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>The source code for the research and education components (Sections 2.1, 2.2., and 2.3) will be saved, stored, and backed up on the UCSB Box. A copy of the code will also be submitted with each of the three planned publications. After the evaluation and refinement of the developed datasets and tools and once the research is completed and published, the final version of the tools and the documentation will be shared on the UCSB’s Dryad Data Repository. The final shareable instructional and teaching materials will also be shared via on a publicly accessible webpage (Scientist Spotlight ) and UCSB Google Drive(workshop materials) and Dryad in pdf format.</t>
+          <t>UCSB Box will be used as the primary means to store and back up all collected input, generated output data sets and code, and educational materials over the course of the project and prior to data sharing. Box provides encryption of data at rest and in-transit, detailed logging of file actions, two-factor authentication, and access review of collaborators. Data will be accessed using Box Drive, which requires full disk encryption, firewall, and an antivirus software in order to install on a local computer. At the end of the project, all shareable data accompanied by the appropriate documentation, metadata, and code will be deposited into Dryad for long-term storage, preservation and accessibility. Deposits submitted to Dryad are curated prior to public release to conform with quality standards and enable future reuse.
+The source code for the research and education components (Sections 2.1, 2.2., and 2.3) will be saved, stored, and backed up on the UCSB Box. A copy of the code will also be submitted with each of the three planned publications. After the evaluation and refinement of the developed datasets and tools and once the research is completed and published, the final version of the tools and the documentation will be shared on the UCSB’s Dryad Data Repository. The final shareable instructional and teaching materials will also be shared via on a publicly accessible webpage (Scientist Spotlight ) and UCSB Google Drive(workshop materials) and Dryad in pdf format.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update sample11 data in Excel export and adjust output summary
</commit_message>
<xml_diff>
--- a/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
+++ b/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
@@ -1097,7 +1097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1119,7 +1119,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1131,46 +1131,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3.3.3 Data Management Plan</t>
+          <t>All participants in the proposed project with access to the numerical codes and computational data will conform closely to NASA policy on preserving and sharing of the research data and gathered in the course of the proposed project. The data acquired and preserved in the context of this proposal will be further governed by UCSB’s policies pertaining to intellectual property, record retention, and data management.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>question.text</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>All participants in the proposed project with access to the numerical codes and computational data will conform closely to NASA policy on preserving and sharing of the research data and gathered in the course of the proposed project. The data acquired and preserved in the context of this proposal will be further governed by UCSB’s policies pertaining to intellectual property, record retention, and data management.</t>
+          <t>3.3.3 Data Management Plan</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
-        <is>
-          <t>3.3.3 Data Management Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
         <is>
           <t>Digital products from this project include: 1) a numerical code that can predict the ADR performance of a magnetic refrigerant based on DFT and DFPT simulation of magnon and phonon properties. The computer code will be published on the open-source website GitHub. PI Liao has published homemade code on GitHub before (https://github.com/nanoengineering/EPW-nano). 2) a numerical code that solves the coupled magnon-phonon Boltzmann transport equations. This software will be written in Python and published and regularly maintained/updated on the open-source website GitHub. 3) Data from first-principles simulations, including magnon and phonon transport properties of selected magnetic materials. Metadata that describes simulation conditions will also be generated, indexed, and archived together with the raw data. Raw simulation data will be carefully curated and archived. The team will archive all data in local computers and a centralized data storage system based on external hard drives, which is synchronized to cloud storage (UCSB provides unlimited Google Drive storage space to researchers). Graduate students participating in this project will be directly responsible for collecting, curating, and archiving the data. They will be trained by PI Liao before the start of the project on the proper protocol of handling data. The stored data will be periodically (at least monthly) inspected by PI Liao. In the event of the departure of key personnel, a written document detailing the content and the condition of the data that they are responsible for should be prepared and data transfer and training should be conducted before the departure.
 We will publish primary results expeditiously in peer-reviewed journals, supported by relevant data in the supplementary documents along with the published papers. Raw data supporting published papers will be made available to the public automatically by depositing the data to the open-access repository Figshare, and the web link will be provided in the published paper. The raw data will be properly annotated and detailed metadata that describes the content, format, organization of the raw data will also be provided to help interpret the raw data. If processed data is used in the publication, the processing procedure will be described in detail in the paper. We will provide full assistance in terms of raw data availability, data processing software and error analysis for other researchers to validate and reproduce our results. We will make peer-reviewed publications from this project all available to the public by depositing the accepted manuscripts to depositories like arXiv and PubMed Central.</t>

</xml_diff>

<commit_message>
Remove sample13 data files and update export notebook to reflect changes in labeled results
</commit_message>
<xml_diff>
--- a/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
+++ b/data/output/pdfplumber_fallback_lightonocr_and_gemma.xlsx
@@ -1463,7 +1463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1509,105 +1509,104 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>question.text</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PI Gu</t>
+          <t>DATA MANAGEMENT PLAN</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PI Gu</t>
+          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The Gu Laboratory is committed to the open sharing and prompt dissemination of all data and resources generated during this project. We will adhere to policies for data management and data sharing set by the NSF.</t>
+          <t>Proteomic Data</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Proteomic Data</t>
+          <t>This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>question.text</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Description
-This project will generate PL-LFQMS profiling data using 13 newly identified PNET proteins as well as KAKU4 and Nup188 as bait. In addition, we will perform substrate-trap PL-LFQMS profiling using two INM PNET proteins to identify potential candidates of PIIs.</t>
+          <t>Proteomic Data</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Archiving and Dissemination</t>
+          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.
+Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Archiving and Dissemination</t>
+          <t>Mutants, Transgenic Lines, and Plasmid Constructs</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>We will make the raw proteomic data available to the public as soon as it has passed quality control criteria in our hands. These data will be deposited to the ProteomeXchange Consortium, which has been set up to provide a coordinated submission of MS proteomics data to the main existing proteomics repositories. All submissions will be set as publicly accessible and include metadata such as transgenic background, bait protein, tag information, controls, etc. Prior to the submission to ProteomeXchange Consortium, the MS data will be maintained both on local hard drives and in the CyVerse Data Store. CyVerse is an NSF-funded cyberinfrastructure initiative dedicated to making large scale computational resource available to a broad range of scientists.
-Normalized MS data, differential enrichment analyses, and associated statistics will be published in peer-reviewed journals and provided as supplementary tables. All analyses and results in papers will also be made freely available upon request following their publication.</t>
+          <t>This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>question.text</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1619,13 +1618,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Description
-This project will generate biological materials of use to the research community, including Arabidopsis transgenic lines expressing fluorescent protein- and proximity biotinylation enzyme-tagged NE proteins, Arabidopsis mutants in which NE-associated genes have been disrupted through CRISPR-based genome editing, as well as plasmid constructs for expression of NE-associated Arabidopsis genes.</t>
+          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
         </is>
       </c>
     </row>
@@ -1637,68 +1635,67 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Archiving and Dissemination</t>
+          <t>Publications</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>question.text</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Archiving and Dissemination</t>
+          <t>Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>answer.text</t>
+          <t>question.text</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>All plasmids constructed will be stored as glycerol stocks in E. coli or A. tumefaciens in -80°C freezer. All transgenic and mutant seeds generated will be maintained in the lab in desiccated environment at room temperature. All above seeds and DNA constructs will also be deposited into publicly accessible repositories, such as Addgene and the Arabidopsis Biological Resource Center (ABRC) at Ohio State University, which will make them available to the research community. They will also be freely available upon request to PI Gu.</t>
+          <t>Publications</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>answer.text</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Publications</t>
+          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>section.description</t>
+          <t>section.title</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Description
-Data obtained in the project will be published promptly. We anticipate that publication of results obtained under this project will start at Year 4 and be completed within a year following the end of the supported period. All data will be made freely available upon request following their publication. There are no anticipated ethical or privacy issues, permission restrictions, or intellectual privacy issues associated with the data following their publication. The PI and the two main participants of this project are also expected to present their findings at two major scientific conferences and other local scientific events.</t>
+          <t>Teaching Curricula</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>section.title</t>
+          <t>section.description</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Archiving and Dissemination</t>
+          <t>Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1707,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Archiving and Dissemination</t>
+          <t>Teaching Curricula</t>
         </is>
       </c>
     </row>
@@ -1721,67 +1718,6 @@
         </is>
       </c>
       <c r="B21" t="inlineStr">
-        <is>
-          <t>In accordance with the University of California Open Access Policy, publications will be uploaded to eScholarship, UC’s open access repository, and publishing platform, to be made available to the public at no charge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Teaching Curricula</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>section.description</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Description
-Lectures on the NE evolution, structure, composition, and function will be developed. In addition, URAP and SPUR student training plans will be generated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>section.title</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Archiving and Dissemination</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>question.text</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Archiving and Dissemination</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>answer.text</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
         <is>
           <t>Lectures, student presentations, data collection, training resources will be maintained online through the UC Berkeley bCourses course management system and backed up online through the unlimited cloud-based storage space offered by Google.</t>
         </is>

</xml_diff>